<commit_message>
fix: dedupe Construction and ITES companies, audit report links
Removed 32 duplicate company entries (same website, different row/name
variant - e.g. "Jacobs Engineering" vs "Jacobs Engineering Group Inc.")
from the live deployment and local dataset: 19 in Construction (109->90),
13 in ITES (109->96). Kept whichever record had a real report URL and/or
richer insights per duplicate group. Removed the same duplicate rows from
the source xlsx files so re-importing won't reintroduce them.

Audited all surviving report URLs (91 total): zero dead links (404/410).
72 SEC EDGAR URLs return 403 to a generic User-Agent but resolve 200 with
a compliant one - confirmed bot-blocking, not dead, matching this repo's
documented link-verification policy (docs/ai-search-workflow.md SS3a).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/PMP_Construction_Companies_USA.xlsx
+++ b/research/PMP_Construction_Companies_USA.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bechtel Group Inc.</t>
+          <t>Fluor Corporation</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -471,26 +471,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>https://www.bechtel.com/</t>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://www.fluor.com/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1124198/000112419826000007/flr-20251231.htm</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bechtel University offers thousands of instructor-led, virtual, online and mobile courses across leadership, technical skills, safety/ethics and languages | Bechtel University is accredited by the International Association for Continuing Education &amp; Training to grant CE credit toward professional certifications | Runs joint early-career/workforce development programs with universities abroad (e.g., Warsaw University of Technology for nuclear, Prince Sultan University in Saudi Arabia)</t>
+          <t>Employees logged over 220,000 hours of training through Fluor University in 2025 | Fluor University offers self-paced, virtual and instructor-led courses spanning discipline-specific technical training to leadership, business acumen and communication | Runs dedicated monthly orientation training for new managers plus a standardized talent-development toolkit</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Bechtel.com Learning &amp; Development page and press releases</t>
+          <t>Fluor Corp FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fluor Corporation</t>
+          <t>Jacobs Engineering Group Inc.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -498,31 +503,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>https://www.fluor.com/</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1124198/000112419826000007/flr-20251231.htm</t>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.jacobs.com/</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/52988/000162828025053316/jec-20250926.htm</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Employees logged over 220,000 hours of training through Fluor University in 2025 | Fluor University offers self-paced, virtual and instructor-led courses spanning discipline-specific technical training to leadership, business acumen and communication | Runs dedicated monthly orientation training for new managers plus a standardized talent-development toolkit</t>
+          <t>Launched Jacobs University, a global L&amp;D hub with four dedicated schools and access to nearly 30,000 training programs, focused partly on AI and digital skills | 97%+ of employees completed the mandatory annual "Living Our Values" training module in fiscal 2025 | Maintains a global graduate development program plus local apprenticeships and 240+ communities of practice for career development</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Fluor Corp FY2025 10-K (SEC EDGAR)</t>
+          <t>Jacobs Engineering FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jacobs Engineering Group Inc.</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -530,31 +535,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>https://www.jacobs.com/</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/52988/000162828025053316/jec-20250926.htm</t>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://aecom.com/</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/868857/000086885725000013/acm-20250930.htm</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Launched Jacobs University, a global L&amp;D hub with four dedicated schools and access to nearly 30,000 training programs, focused partly on AI and digital skills | 97%+ of employees completed the mandatory annual "Living Our Values" training module in fiscal 2025 | Maintains a global graduate development program plus local apprenticeships and 240+ communities of practice for career development</t>
+          <t>Operates Global Technical Academies delivering structured/self-directed technical training on key markets and practices | "Leadership at all Levels" program spans early-career/graduate programs, manager training, and executive coaching built on four Leadership Capability pillars | Technical Practice Network connects professionals daily for peer learning across global offices</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Jacobs Engineering FY2025 10-K (SEC EDGAR)</t>
+          <t>AECOM FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>Turner Construction Company</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -562,31 +567,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>https://aecom.com/</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/868857/000086885725000013/acm-20250930.htm</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://www.turnerconstruction.com/</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Operates Global Technical Academies delivering structured/self-directed technical training on key markets and practices | "Leadership at all Levels" program spans early-career/graduate programs, manager training, and executive coaching built on four Leadership Capability pillars | Technical Practice Network connects professionals daily for peer learning across global offices</t>
+          <t>Turner University is Turner's corporate-based university offering construction-specific professional development for employees | Turner School of Construction Management (TSCM), running since 1969, is a free program building project management, estimating, scheduling and finance skills | Construction Ready Program supports workforce pipeline development in local markets</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AECOM FY2025 10-K (SEC EDGAR)</t>
+          <t>Turner Construction insights pages, turnerconstruction.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Turner Construction Company</t>
+          <t>Kiewit Corporation</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -594,26 +594,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>https://www.turnerconstruction.com/</t>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://www.kiewit.com/</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Turner University is Turner's corporate-based university offering construction-specific professional development for employees | Turner School of Construction Management (TSCM), running since 1969, is a free program building project management, estimating, scheduling and finance skills | Construction Ready Program supports workforce pipeline development in local markets</t>
+          <t>Kiewit University (est. 2007) and a dedicated Training Center host corporate training across operations management, scheduling, formwork, design integration and craft skills, serving 6,000+ learners annually | Kiewit spends an average of $7,500 per employee per year on training and career development, above the national industry average | More than 500 internal managers deliver training annually under a "NextGen" hybrid/flipped-classroom model</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Turner Construction insights pages, turnerconstruction.com</t>
+          <t>Kiewit Newsroom/Kieways articles, kiewit.com</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PCL Construction Enterprises Inc.</t>
+          <t>The Whiting-Turner Contracting Company</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -621,26 +621,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>https://www.pcl.com/</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://www.whiting-turner.com/</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PCL College of Construction is PCL's in-house professional development arm covering technical, leadership and behavioral competency training | E3 Leadership Certification Program (education, exposure, experience) has produced 1,000+ graduates since launching in 2017 | Accelerated Superintendent Development Program targets high-potential field employees; Learning Road Maps help staff plan individualized training paths</t>
+          <t>"Whiting-Turner 101" onboarding program trains new hires and interns on company processes, culture and technology | Offers tuition reimbursement up to $5,250/year for job-related coursework | Supports OSHA 30 and other personal certifications plus a formal mentorship program pairing employees with peer/leader networks</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PCL Construction careers/insights pages, pcl.com</t>
+          <t>Whiting-Turner careers pages, whiting-turner.com</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kiewit Corporation</t>
+          <t>DPR Construction</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -648,26 +648,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>https://www.kiewit.com/</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://www.dpr.com/</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Kiewit University (est. 2007) and a dedicated Training Center host corporate training across operations management, scheduling, formwork, design integration and craft skills, serving 6,000+ learners annually | Kiewit spends an average of $7,500 per employee per year on training and career development, above the national industry average | More than 500 internal managers deliver training annually under a "NextGen" hybrid/flipped-classroom model</t>
+          <t>Builder Development Program is a structured, cohort-based launchpad for early-career employees | Foremen Development Program is a paid week-long leadership/safety/planning training; 95% of participants reported better role understanding afterward | Craft Apprenticeship Program is NCCER-certified, covering construction math, blueprint reading and trade-specific learning paths</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Kiewit Newsroom/Kieways articles, kiewit.com</t>
+          <t>DPR Construction careers/blog pages, dpr.com</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The Whiting-Turner Contracting Company</t>
+          <t>Gilbane Building Company</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -675,26 +675,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>https://www.whiting-turner.com/</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://www.gilbaneco.com/</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>"Whiting-Turner 101" onboarding program trains new hires and interns on company processes, culture and technology | Offers tuition reimbursement up to $5,250/year for job-related coursework | Supports OSHA 30 and other personal certifications plus a formal mentorship program pairing employees with peer/leader networks</t>
+          <t>Gilbane University, established in 2000, is the firm's flagship internal training organization with 500+ courses spanning construction management, safety, leadership and software systems | Ranked 28th in Training magazine's 2025 Training APEX Awards, having been recognized as a top training organization 17 times | Gilbane Leadership Development Program (GLDP) is a year-long program including a multiday retreat at Babson University for future business-unit leaders</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Whiting-Turner careers pages, whiting-turner.com</t>
+          <t>Gilbane Building Company news/careers pages, gilbaneco.com</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DPR Construction</t>
+          <t>Hensel Phelps</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -702,26 +702,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
-        <is>
-          <t>https://www.dpr.com/</t>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://www.henselphelps.com/</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Builder Development Program is a structured, cohort-based launchpad for early-career employees | Foremen Development Program is a paid week-long leadership/safety/planning training; 95% of participants reported better role understanding afterward | Craft Apprenticeship Program is NCCER-certified, covering construction math, blueprint reading and trade-specific learning paths</t>
+          <t>Broad training program spans safety/skills training to leadership development via blended instructor-led, online and one-on-one sessions | LeaderFlow Training Development Program is a seven-month nonprofit-partnered leadership curriculum covering strategic thinking, communication and team empowerment | Also runs an Emerging Leaders Seminar and a Women's Leadership Seminar; average employee tenure is 13 years</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>DPR Construction careers/blog pages, dpr.com</t>
+          <t>Hensel Phelps careers/training pages, henselphelps.com</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Gilbane Building Company</t>
+          <t>Skanska USA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -729,26 +729,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>https://www.gilbaneco.com/</t>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://www.usa.skanska.com/</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Gilbane University, established in 2000, is the firm's flagship internal training organization with 500+ courses spanning construction management, safety, leadership and software systems | Ranked 28th in Training magazine's 2025 Training APEX Awards, having been recognized as a top training organization 17 times | Gilbane Leadership Development Program (GLDP) is a year-long program including a multiday retreat at Babson University for future business-unit leaders</t>
+          <t>Skanska Learning Center (SLC) delivers role-specific training company-wide | Core Competency Training Program (CCTP) is a two-year rotational program for entry-level civil engineers; a separate 15-month Superintendent Development Program (since 2021) moves craft foremen into superintendent roles | Excellence in Construction Leadership Program (ECLP) combines project-management/client-relations training with mentorship; company also offers financial support toward degrees and professional licenses</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Gilbane Building Company news/careers pages, gilbaneco.com</t>
+          <t>Skanska USA careers pages, usa.skanska.com</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hensel Phelps</t>
+          <t>Lendlease</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -756,26 +756,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
-        <is>
-          <t>https://www.henselphelps.com/</t>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://www.lendlease.com/</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Broad training program spans safety/skills training to leadership development via blended instructor-led, online and one-on-one sessions | LeaderFlow Training Development Program is a seven-month nonprofit-partnered leadership curriculum covering strategic thinking, communication and team empowerment | Also runs an Emerging Leaders Seminar and a Women's Leadership Seminar; average employee tenure is 13 years</t>
+          <t>Springboard is Lendlease's flagship global development program (launched 1998) blending personal development, wellbeing and community involvement into employee learning | Internal survey found 97% of staff agree Lendlease is committed to employee development | Sustainability Framework Goals explicitly commit to training and developing people as part of ESG reporting (tracked via annual ESG Databook since 2021)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Hensel Phelps careers/training pages, henselphelps.com</t>
+          <t>Lendlease sustainability pages and case studies, lendlease.com</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Skanska USA</t>
+          <t>Balfour Beatty US</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -783,26 +783,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
-        <is>
-          <t>https://www.usa.skanska.com/</t>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://www.balfourbeattyus.com/</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Skanska Learning Center (SLC) delivers role-specific training company-wide | Core Competency Training Program (CCTP) is a two-year rotational program for entry-level civil engineers; a separate 15-month Superintendent Development Program (since 2021) moves craft foremen into superintendent roles | Excellence in Construction Leadership Program (ECLP) combines project-management/client-relations training with mentorship; company also offers financial support toward degrees and professional licenses</t>
+          <t>Balfour Beatty Academy applies a 70:20:10 development model covering technical expertise, personal skills and professional qualifications | Structured apprenticeship pathways (Intermediate/Advanced/Higher/Degree level) typically run two years and lead to industry-recognized qualifications | Apprentices are paired with mentors and joined into a peer-support network alongside line-manager development plans</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Skanska USA careers pages, usa.skanska.com</t>
+          <t>Balfour Beatty careers pages, balfourbeattyus.com</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Lendlease</t>
+          <t>Lennar Corporation</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -810,26 +810,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lendlease.com/</t>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://www.lennar.com/</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/920760/000162828026003870/len-20251130.htm</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Springboard is Lendlease's flagship global development program (launched 1998) blending personal development, wellbeing and community involvement into employee learning | Internal survey found 97% of staff agree Lendlease is committed to employee development | Sustainability Framework Goals explicitly commit to training and developing people as part of ESG reporting (tracked via annual ESG Databook since 2021)</t>
+          <t>Leadership Development Program delivered in partnership with Harvard Business School Publishing combines live instructor-led virtual sessions with individual assignments | Lennar Management Training (powered by Harvard ManageMentor) offers self-paced business-management courses available to all associates | Future Builders Program gives recent graduates structured rotational exposure to the homebuilding business</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Lendlease sustainability pages and case studies, lendlease.com</t>
+          <t>Lennar FY2025 10-K and careers.lennar.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Balfour Beatty US</t>
+          <t>D.R. Horton Inc.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -837,26 +842,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
-        <is>
-          <t>https://www.balfourbeattyus.com/</t>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://www.drhorton.com/</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/882184/000088218425000081/dhi-20250930.htm</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Balfour Beatty Academy applies a 70:20:10 development model covering technical expertise, personal skills and professional qualifications | Structured apprenticeship pathways (Intermediate/Advanced/Higher/Degree level) typically run two years and lead to industry-recognized qualifications | Apprentices are paired with mentors and joined into a peer-support network alongside line-manager development plans</t>
+          <t>Leadership Development Program provides internal training to prepare future leaders across all operating areas; 18 employees were placed into new homebuilding markets via internal mobility in fiscal 2025 | Runs specialized functional training for purchasing, construction, sales and financial-management staff | Provides third-party OSHA certification training for field personnel plus mandatory cybersecurity/compliance training</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Balfour Beatty careers pages, balfourbeattyus.com</t>
+          <t>D.R. Horton FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Toll Brothers Inc.</t>
+          <t>NVR Inc.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -864,31 +874,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tollbrothers.com/</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/794170/000079417025000112/tol-20251031.htm</t>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.nvrinc.com/</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/906163/000090616326000018/nvr-20251231.htm</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Toll Brothers University and its Talent Development Team run technical and soft-skills courses, including specialized onboarding for new people leaders, Sales and Construction staff | National Production Training Program is split into five curriculums covering technical, managerial, leadership, personal-development and field-proficiency skills | Offers tuition reimbursement for work-related coursework and a nine-month Management Associate rotational program</t>
+          <t>offers structured onboarding and mentor-pairing for new hires, given its stated practice of promoting roughly 80% of managers from within with average manager tenure of 20 years | provides cross-functional job rotation opportunities for employees to broaden skills across departments | maintains division-specific technical training blending online modules with hands-on field coaching</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Toll Brothers FY2025 10-K and Toll Career Center</t>
+          <t>NVR FY2025 10-K plus nvrcareers.com â€” no named formal L&amp;D program/budget disclosed</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lennar Corporation</t>
+          <t>PulteGroup Inc.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -896,31 +906,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lennar.com/</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/920760/000162828026003870/len-20251130.htm</t>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.pultegroupinc.com/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/822416/000082241626000007/phm-20251231.htm</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Leadership Development Program delivered in partnership with Harvard Business School Publishing combines live instructor-led virtual sessions with individual assignments | Lennar Management Training (powered by Harvard ManageMentor) offers self-paced business-management courses available to all associates | Future Builders Program gives recent graduates structured rotational exposure to the homebuilding business</t>
+          <t>Runs "Breaking Ground," a structured onboarding program pairing every new hire with a mentor | Certified Field Trainer initiative supports new field/operational hires for up to six months | Maintains a dedicated VP of Leadership Development role overseeing a leadership-development pipeline and expanding D&amp;I training</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Lennar FY2025 10-K and careers.lennar.com</t>
+          <t>PulteGroup FY2025 10-K and newsroom.pultegroup.com</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>D.R. Horton Inc.</t>
+          <t>Meritage Homes Corporation</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -928,31 +938,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C18" s="1" t="inlineStr">
-        <is>
-          <t>https://www.drhorton.com/</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/882184/000088218425000081/dhi-20250930.htm</t>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.meritagehomes.com/</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/833079/000083307926000010/mth-20251231.htm</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Leadership Development Program provides internal training to prepare future leaders across all operating areas; 18 employees were placed into new homebuilding markets via internal mobility in fiscal 2025 | Runs specialized functional training for purchasing, construction, sales and financial-management staff | Provides third-party OSHA certification training for field personnel plus mandatory cybersecurity/compliance training</t>
+          <t>1,860 full-time employees as of Dec 31, 2025, spanning management, sales, and construction/warranty operations | Formal talent recognition and succession-planning model designed to identify high-potential employees and build advancement roadmaps within the company | Comprehensive benefits package includes tuition reimbursement plus wellness, caregiving, and employee-assistance programs to support ongoing employee development</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>D.R. Horton FY2025 10-K (SEC EDGAR)</t>
+          <t>Meritage Homes FY2025 10-K, Human Capital section (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NVR Inc.</t>
+          <t>KB Home</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -960,31 +970,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C19" s="1" t="inlineStr">
-        <is>
-          <t>https://www.nvrinc.com/</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/906163/000090616326000018/nvr-20251231.htm</t>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.kbhome.com/</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/795266/000079526626000017/kbh-20251130.htm</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>offers structured onboarding and mentor-pairing for new hires, given its stated practice of promoting roughly 80% of managers from within with average manager tenure of 20 years | provides cross-functional job rotation opportunities for employees to broaden skills across departments | maintains division-specific technical training blending online modules with hands-on field coaching</t>
+          <t>Runs KBU, an internet-based enterprise learning platform with a library of roughly 412 self-directed and instructor-led courses plus 50 leadership/managerial training topics | Team members completed more than 28,169 courses in FY2023, averaging about 13 courses per employee company-wide | 6-session 'Managing Essentials' management training series graduated 69 managers in FY2023, bringing total graduates to over 413 across the past decade; tuition reimbursement offered as a career-development benefit</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>NVR FY2025 10-K plus nvrcareers.com â€” no named formal L&amp;D program/budget disclosed</t>
+          <t>KB Home FY2023 10-K, Human Capital section (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PulteGroup Inc.</t>
+          <t>Tri Pointe Homes Inc.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -992,31 +1002,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>https://www.pultegroupinc.com/</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/822416/000082241626000007/phm-20251231.htm</t>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://www.tripointehomes.com/</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=TPH</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Runs "Breaking Ground," a structured onboarding program pairing every new hire with a mentor | Certified Field Trainer initiative supports new field/operational hires for up to six months | Maintains a dedicated VP of Leadership Development role overseeing a leadership-development pipeline and expanding D&amp;I training</t>
+          <t>Operates 'Blueprint,' a proprietary online learning center where team members build self-paced, curated learning paths | Pairs a job-specific onboarding program with Blueprint to accelerate new hires' ramp-up and social integration | Launched the 'Cornerstone Club' in 2025, an internal ambassador group focused on development, mentoring, and campus/military recruiting outreach; workforce of roughly 1,400 team members; named to Fortune's Best Workplaces in Construction for four consecutive years</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>PulteGroup FY2025 10-K and newsroom.pultegroup.com</t>
+          <t>Tri Pointe Homes 10-K/investor disclosures and company press releases</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Taylor Morrison Home Corporation</t>
+          <t>The Ryland Group Inc.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1024,31 +1034,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
-        <is>
-          <t>https://www.taylormorrison.com/</t>
-        </is>
-      </c>
-      <c r="D21" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1562476/000162828026009030/tmhc-20251231.htm</t>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.ryland.com/</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Learning management system gives employees access to more than 5,000 online courses plus tailored leadership-development programs by career stage | Offers tuition reimbursement as part of its standard benefits package | Requires mandatory ongoing cybersecurity training and additional health/safety training for construction and field personnel</t>
+          <t>The Ryland Group is defunct as an independent entity â€” it merged with Standard Pacific Corp in October 2015 to form CalAtlantic Group, and CalAtlantic was then acquired by Lennar Corporation in January 2018, fully retiring the Ryland brand | any legacy Ryland training or leadership-development programs would have been absorbed into CalAtlantic's and later Lennar's own corporate L&amp;D infrastructure | as a pre-2015 public homebuilder, Ryland's historical 10-Ks would have included only generic human-capital language typical of that era rather than detailed named-program disclosures</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Taylor Morrison FY2025 10-K (SEC EDGAR)</t>
+          <t>Defunct; merged into CalAtlantic (2015) then Lennar (2018) per SEC 8-K/425 merger filings</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Meritage Homes Corporation</t>
+          <t>Standard Pacific Corp.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1056,31 +1061,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C22" s="1" t="inlineStr">
-        <is>
-          <t>https://www.meritagehomes.com/</t>
-        </is>
-      </c>
-      <c r="D22" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/833079/000083307926000010/mth-20251231.htm</t>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://www.standardpacifichomes.com/</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1,860 full-time employees as of Dec 31, 2025, spanning management, sales, and construction/warranty operations | Formal talent recognition and succession-planning model designed to identify high-potential employees and build advancement roadmaps within the company | Comprehensive benefits package includes tuition reimbursement plus wellness, caregiving, and employee-assistance programs to support ongoing employee development</t>
+          <t>Standard Pacific Corp. no longer exists as an independent company â€” it merged with The Ryland Group on October 1, 2015 to form CalAtlantic Group, Inc. | any pre-2015 employee training or L&amp;D programs were absorbed into CalAtlantic's HR structure, which itself was later acquired by Lennar in February 2018 | as a defunct entity with no active careers site or investor relations, there is no current, targetable training/L&amp;D budget or program to reference for outreach</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Meritage Homes FY2025 10-K, Human Capital section (SEC EDGAR)</t>
+          <t>Merged into CalAtlantic Group (Oct 2015); CalAtlantic later merged into Lennar (2018) per SEC 8-K filings</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>KB Home</t>
+          <t>Centex Corporation</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1088,31 +1088,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C23" s="1" t="inlineStr">
-        <is>
-          <t>https://www.kbhome.com/</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/795266/000079526626000017/kbh-20251130.htm</t>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.centex.com/</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Runs KBU, an internet-based enterprise learning platform with a library of roughly 412 self-directed and instructor-led courses plus 50 leadership/managerial training topics | Team members completed more than 28,169 courses in FY2023, averaging about 13 courses per employee company-wide | 6-session 'Managing Essentials' management training series graduated 69 managers in FY2023, bringing total graduates to over 413 across the past decade; tuition reimbursement offered as a career-development benefit</t>
+          <t>Centex Corporation no longer exists as an independent company â€” it merged into Pulte Homes, Inc. (now PulteGroup) in a stock-for-stock deal valued at $3.1 billion, completed August 2009 | the combined company became the largest U.S. homebuilder at the time, so any legacy Centex training infrastructure was folded into Pulte's corporate L&amp;D function | no standalone careers page, 10-K, or ESG report exists for Centex today, so training/L&amp;D outreach would need to target PulteGroup directly instead</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>KB Home FY2023 10-K, Human Capital section (SEC EDGAR)</t>
+          <t>Merged into Pulte Homes/PulteGroup (Aug 2009) per SEC 8-K/425 filings</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>M.D.C. Holdings Inc.</t>
+          <t>The Mosaic Company</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1120,31 +1115,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C24" s="1" t="inlineStr">
-        <is>
-          <t>https://www.richmondamerican.com/</t>
-        </is>
-      </c>
-      <c r="D24" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=MDC</t>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://www.mosaicco.com/</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1285785/000128578526000017/mos-20251231.htm</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>About 1,826 employees as of Dec 31, 2024 (up from 1,760 in 2023), with training cited as a core human-capital investment area | Offers ongoing training and development through online resources, job shadowing, and mentoring programs across career paths | Requires annual compliance training under its Code of Conduct, including mandatory instruction on preventing and reporting workplace discrimination</t>
+          <t>FY2025 10-K Human Capital section highlights executive-led Employee Inclusion Networks (EINs) open to all employees, expanded following insights from a 2024 companywide Voice of the Employee survey | Company states "ongoing awareness and education continue to be a cornerstone" of its inclusive-culture strategy, indicating structured internal training/awareness programming | Mosaic annually evaluates pay equity and compensation practices under a formal pay-for-performance framework tied to its broader talent/retention strategy</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>M.D.C. Holdings FY2023/2024 10-K, Human Capital section; note MDC Holdings was acquired by Sekisui House in 2024 and no longer files independently, so this is the last available public disclosure</t>
+          <t>The Mosaic Company FY2025 Form 10-K, Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tri Pointe Homes Inc.</t>
+          <t>Quanta Services Inc.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1152,31 +1147,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tripointehomes.com/</t>
-        </is>
-      </c>
-      <c r="D25" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=TPH</t>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://www.quantaservices.com/</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1050915/000105091526000006/pwr-20251231.htm</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Operates 'Blueprint,' a proprietary online learning center where team members build self-paced, curated learning paths | Pairs a job-specific onboarding program with Blueprint to accelerate new hires' ramp-up and social integration | Launched the 'Cornerstone Club' in 2025, an internal ambassador group focused on development, mentoring, and campus/military recruiting outreach; workforce of roughly 1,400 team members; named to Fortune's Best Workplaces in Construction for four consecutive years</t>
+          <t>Operates the Quanta Advanced Training Center, a 2,300-acre campus providing hands-on instruction from master trainers in real-world-job-site-style environments for safety, skills, and certifications | Has trained over 50,000 team members across multiple training and apprenticeship programs, including a workforce-development partnership with Sam Houston State University established in 2016 | Runs a Cornerstone LMS-based "Crew Leadership Level 2" program for newly promoted leaders and operates the electric utility industry's only in-house aviation/helicopter training program</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Tri Pointe Homes 10-K/investor disclosures and company press releases</t>
+          <t>Quanta Services corporate training pages (quantaservices.com/training); FY2025 10-K</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>The Ryland Group Inc.</t>
+          <t>Emerson Electric Co.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1184,26 +1179,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ryland.com/</t>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://www.emerson.com/</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/32604/000003260425000087/emr-20250930.htm</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>The Ryland Group is defunct as an independent entity â€” it merged with Standard Pacific Corp in October 2015 to form CalAtlantic Group, and CalAtlantic was then acquired by Lennar Corporation in January 2018, fully retiring the Ryland brand | any legacy Ryland training or leadership-development programs would have been absorbed into CalAtlantic's and later Lennar's own corporate L&amp;D infrastructure | as a pre-2015 public homebuilder, Ryland's historical 10-Ks would have included only generic human-capital language typical of that era rather than detailed named-program disclosures</t>
+          <t>10-K Human Capital section states Emerson "supports and develops its employees through global training and development programs that build and strengthen employees' leadership and professional skills," including intensive programs for both new and established leaders | Company partners with educational institutions to help prepare current and future workers with needed skills, and offers tuition reimbursement as part of its standard benefits package | Implemented a globally consistent digital continuous-listening/engagement survey strategy in 2023; in FY2025, 91% of employees participated and overall engagement score held steady at 79%</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Defunct; merged into CalAtlantic (2015) then Lennar (2018) per SEC 8-K/425 merger filings</t>
+          <t>Emerson Electric Co. FY2025 Form 10-K, Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Standard Pacific Corp.</t>
+          <t>Primoris Services Corporation</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1211,26 +1211,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>https://www.standardpacifichomes.com/</t>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.prim.com/</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1361538/000110465926018677/prim-20251231x10k.htm</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Standard Pacific Corp. no longer exists as an independent company â€” it merged with The Ryland Group on October 1, 2015 to form CalAtlantic Group, Inc. | any pre-2015 employee training or L&amp;D programs were absorbed into CalAtlantic's HR structure, which itself was later acquired by Lennar in February 2018 | as a defunct entity with no active careers site or investor relations, there is no current, targetable training/L&amp;D budget or program to reference for outreach</t>
+          <t>Runs five cornerstone leadership development programs -- Foreman Foundations, Extreme Ownership, Hunt for Leadership Success, Next Level Leadership, and The Leadership Experience -- progressing employees from crew leader to strategic leadership skills | Maintains company-owned training facilities for on- and off-site skills training, including sites that train electrical apprentices through to journeyman status | Tracks safety metrics reviewed monthly by senior management, with site leadership evaluated on safety-culture performance</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Merged into CalAtlantic Group (Oct 2015); CalAtlantic later merged into Lennar (2018) per SEC 8-K filings</t>
+          <t>Primoris Services Corp FY2025 10-K (SEC), Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Centex Corporation</t>
+          <t>Granite Construction Incorporated</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1238,26 +1243,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C28" s="1" t="inlineStr">
-        <is>
-          <t>https://www.centex.com/</t>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://www.graniteconstruction.com/</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/861459/000086145926000004/gva-20251231.htm</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Centex Corporation no longer exists as an independent company â€” it merged into Pulte Homes, Inc. (now PulteGroup) in a stock-for-stock deal valued at $3.1 billion, completed August 2009 | the combined company became the largest U.S. homebuilder at the time, so any legacy Centex training infrastructure was folded into Pulte's corporate L&amp;D function | no standalone careers page, 10-K, or ESG report exists for Centex today, so training/L&amp;D outreach would need to target PulteGroup directly instead</t>
+          <t>Runs "Granite University," an internal L&amp;D function with dedicated learning specialists, an online learning management system for course tracking, and a 5,000-square-foot training facility with multiple classrooms and a computer lab | Course catalog spans classroom instruction, interactive eLearning, and desktop-based content covering technical and career-development topics | Actively promotes continued external education to help employees build certifications and degrees alongside internal training</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Merged into Pulte Homes/PulteGroup (Aug 2009) per SEC 8-K/425 filings</t>
+          <t>Granite Construction careers site (granitenet.com/careers/granite-university)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>The Mosaic Company</t>
+          <t>Tetra Tech Inc.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1265,31 +1275,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C29" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mosaicco.com/</t>
-        </is>
-      </c>
-      <c r="D29" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1285785/000128578526000017/mos-20251231.htm</t>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.tetratech.com/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/831641/000083164125000032/ttek-20250928.htm</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>FY2025 10-K Human Capital section highlights executive-led Employee Inclusion Networks (EINs) open to all employees, expanded following insights from a 2024 companywide Voice of the Employee survey | Company states "ongoing awareness and education continue to be a cornerstone" of its inclusive-culture strategy, indicating structured internal training/awareness programming | Mosaic annually evaluates pay equity and compensation practices under a formal pay-for-performance framework tied to its broader talent/retention strategy</t>
+          <t>Tetra Tech's Learning Hub delivers project management, leadership development, and technical skills training via online courses, virtual workshops, and in-person events for 25,000+ staff worldwide | Thousands of employees have completed Tetra Tech's Project Management Training program covering all phases of the project life cycle | Company offers accredited certification programs (IACET, APMG International, ANSI) and runs IP3 (Institute for Public-Private Partnerships), a Tetra Tech company providing PPP certification training</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>The Mosaic Company FY2025 Form 10-K, Human Capital section</t>
+          <t>Tetra Tech FY2025 10-K Human Capital section + tetratech.com Learning and Development pages</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Quanta Services Inc.</t>
+          <t>Arcadis U.S. Inc.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1297,31 +1307,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
-        <is>
-          <t>https://www.quantaservices.com/</t>
-        </is>
-      </c>
-      <c r="D30" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1050915/000105091526000006/pwr-20251231.htm</t>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://www.arcadis.com/</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Operates the Quanta Advanced Training Center, a 2,300-acre campus providing hands-on instruction from master trainers in real-world-job-site-style environments for safety, skills, and certifications | Has trained over 50,000 team members across multiple training and apprenticeship programs, including a workforce-development partnership with Sam Houston State University established in 2016 | Runs a Cornerstone LMS-based "Crew Leadership Level 2" program for newly promoted leaders and operates the electric utility industry's only in-house aviation/helicopter training program</t>
+          <t>Arcadis Energy Transition Academy targets training or recruiting 2,500+ 'Arcadian' energy experts by 2027, backed by an in-house online platform (ETA@Home) with curated technical modules | Citizen Development program is a 3-month upskilling track in data, cloud, security, AI, and software development that produced a 40% increase in tech proficiency within 90 days | Arcadis Talent Academy is a 6-month paid-job-track program combining real project experience with language and soft-skills training; company also partnered with Pluralsight Skills for digital-fluency upskilling</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Quanta Services corporate training pages (quantaservices.com/training); FY2025 10-K</t>
+          <t>Arcadis.com newsroom, Arcadis 2024 Annual Integrated Report, Pluralsight case study</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Emerson Electric Co.</t>
+          <t>Black &amp; Veatch</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1329,31 +1334,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C31" s="1" t="inlineStr">
-        <is>
-          <t>https://www.emerson.com/</t>
-        </is>
-      </c>
-      <c r="D31" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/32604/000003260425000087/emr-20250930.htm</t>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://www.bv.com/</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>10-K Human Capital section states Emerson "supports and develops its employees through global training and development programs that build and strengthen employees' leadership and professional skills," including intensive programs for both new and established leaders | Company partners with educational institutions to help prepare current and future workers with needed skills, and offers tuition reimbursement as part of its standard benefits package | Implemented a globally consistent digital continuous-listening/engagement survey strategy in 2023; in FY2025, 91% of employees participated and overall engagement score held steady at 79%</t>
+          <t>Black &amp; Veatch offers tuition assistance for full-time employee-owners, rated 4.0/5 by employees on Glassdoor for this benefit | ENT Accelerator Program is a full-time paid entry-level training track where trainees start earning pay and benefits on day one of class | As an employee-owned firm, the company bundles professional development with 401(k) match, professional-society support, and wellbeing programs as part of its 'people first' Total Rewards approach</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Emerson Electric Co. FY2025 Form 10-K, Human Capital section</t>
+          <t>Glassdoor Black &amp; Veatch benefits page, bv.com Early Careers/ENT Accelerator Program page</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MasTec Inc.</t>
+          <t>CH2M</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1361,31 +1361,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C32" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mastec.com/</t>
-        </is>
-      </c>
-      <c r="D32" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/15615/000001561526000020/mtz-20251231.htm</t>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://www.ch2m.com/</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Runs regular safety training and skill-level improvement programs including new-employee safety orientation, safety leadership training for front-line leaders, OSHA construction outreach training, and defensive driving/DOT training | Operates under a company-wide "Zero Harm" safety culture instilled in all ~36,000 employees | Workforce includes ~9,000 unionized employees, many trained via union apprenticeship/journeyman pipelines tied to craft trades</t>
+          <t>CH2M HILL no longer exists as a standalone company â€” Jacobs Engineering completed its acquisition on December 15, 2017 for ~$1.8B cash plus ~$1.4B of Jacobs stock, fully absorbing CH2M's workforce and operations | any legacy CH2M training programs (e.g., project management and technical certification tracks) were folded into Jacobs' own learning infrastructure post-merger | successor Jacobs Engineering runs enterprise-wide learning and leadership-development programs, including project-management and technical certification support</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>MasTec FY2025 10-K (SEC), Human Capital section</t>
+          <t>SEC EDGAR Jacobs Engineering S-4/10-Q filings on the 2017 CH2M acquisition</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Primoris Services Corporation</t>
+          <t>Burns &amp; McDonnell</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1393,31 +1388,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C33" s="1" t="inlineStr">
-        <is>
-          <t>https://www.prim.com/</t>
-        </is>
-      </c>
-      <c r="D33" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1361538/000110465926018677/prim-20251231x10k.htm</t>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://www.burnsmcd.com/</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Runs five cornerstone leadership development programs -- Foreman Foundations, Extreme Ownership, Hunt for Leadership Success, Next Level Leadership, and The Leadership Experience -- progressing employees from crew leader to strategic leadership skills | Maintains company-owned training facilities for on- and off-site skills training, including sites that train electrical apprentices through to journeyman status | Tracks safety metrics reviewed monthly by senior management, with site leadership evaluated on safety-culture performance</t>
+          <t>Burns &amp; McDonnell delivers roughly 2,500 in-house company-led development classes per year spanning technical, computer, safety, and professional-development topics, taught online, in-person, and on-demand | Tuition reimbursement covers up to the IRS non-taxable limit annually for Bachelor's study and up to $10,000/year for Master's study, available to full-time employee-owners after 6 months of service | Employee-owners can earn Professional Development Hours (PDH) from completed courses, and the company pays professional/technical society membership dues plus offers career-counseling through its Professional Development Department</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Primoris Services Corp FY2025 10-K (SEC), Human Capital section</t>
+          <t>burnsmcd.com Training &amp; Development careers page; Glassdoor Burns &amp; McDonnell Tuition Assistance benefit page</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Granite Construction Incorporated</t>
+          <t>HNTB Corporation</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1425,31 +1415,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
-        <is>
-          <t>https://www.graniteconstruction.com/</t>
-        </is>
-      </c>
-      <c r="D34" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/861459/000086145926000004/gva-20251231.htm</t>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://www.hntb.com/</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Runs "Granite University," an internal L&amp;D function with dedicated learning specialists, an online learning management system for course tracking, and a 5,000-square-foot training facility with multiple classrooms and a computer lab | Course catalog spans classroom instruction, interactive eLearning, and desktop-based content covering technical and career-development topics | Actively promotes continued external education to help employees build certifications and degrees alongside internal training</t>
+          <t>Formal mentorship program pairs mentors and mentees for professional growth, plus tuition reimbursement/financial assistance for continuing education | HNTB Fellows Program recognizes top technical leadership, mentoring, and consulting achievement company-wide | Learning &amp; Development team manages training via Workday Learning, offering leadership courses, workshops, webinars, and structured onboarding for new hires and interns</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Granite Construction careers site (granitenet.com/careers/granite-university)</t>
+          <t>HNTB corporate site, careers/FAQ pages</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MYR Group Inc.</t>
+          <t>Toll Brothers</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1457,31 +1442,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C35" s="1" t="inlineStr">
-        <is>
-          <t>https://www.myrgroup.com/</t>
-        </is>
-      </c>
-      <c r="D35" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/700923/000070092326000007/myrg-20251231.htm</t>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://www.tollbrothers.com/</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/794170/000079417025000112/tol-20251031.htm</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Non-union subsidiary Great Southwestern Construction runs a paid electrical-apprenticeship program at a dedicated training facility in Alvarado, Texas, combining work-based learning with related classroom instruction | Most MYR Group subsidiaries operate in IBEW jurisdictions and participate in national and local Joint Apprenticeship Training Committees (JATCs) for electrical trade certification | Partners on community workforce-development initiatives (e.g., with the Detroit Public Lighting Authority and IBEW Local 17) to widen access to electrical-trade training</t>
+          <t>FY2025 10-K confirms mandatory annual training for all employees on preventing/reporting workplace discrimination as part of code of conduct | Company (approx. 4,900 full-time employees) states it focuses significant resources on attracting, developing, and retaining talented staff, monitored via engagement/satisfaction surveys | Sustainability reporting references leadership development, diversity training, and mentorship programs, though specific training-hour metrics are not publicly broken out</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>MYR Group corporate site / news releases (myrgroup.com)</t>
+          <t>Toll Brothers FY2025 10-K (SEC EDGAR) human capital section + tollbrothers.com/sustainability</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ameresco Inc.</t>
+          <t>MasTec</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1489,31 +1474,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C36" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ameresco.com/</t>
-        </is>
-      </c>
-      <c r="D36" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1488139/000162828026013574/amrc_20251231x10-k.htm</t>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://www.mastec.com/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/15615/000001561526000020/mtz-20251231.htm</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>offers technical/certification training for energy engineers and project staff (e.g., PE, CEM, LEED credentials) given its energy-services/ESCO business model | provides structured onboarding and role-based technical development programs for its ~1,500+ employees across US, Canada, UK and Italy offices | Encourages employee community engagement through paid volunteer/community-service days as part of its broader people program</t>
+          <t>Provides regular safety and skill-level training including safety leadership training for front-line leaders, OSHA construction outreach training, and operator qualification/electric worker training | Runs ongoing internally-developed educational programs combining classroom and field training to build technical and management skills | ~36,000 employees as of Dec 2025, with training/career development framed as a core retention and attraction strategy under its 'Zero Harm' safety culture</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Ameresco 10-K filings (SEC) Human Capital section; no specific training-program figures found</t>
+          <t>MasTec FY2025 10-K (SEC EDGAR, mtz-20251231.htm) human capital section</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tetra Tech Inc.</t>
+          <t>MDU Resources</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1521,31 +1506,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C37" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tetratech.com/</t>
-        </is>
-      </c>
-      <c r="D37" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/831641/000083164125000032/ttek-20250928.htm</t>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://www.mdu.com/</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/67716/000006771626000014/mdu-20251231.htm</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Tetra Tech's Learning Hub delivers project management, leadership development, and technical skills training via online courses, virtual workshops, and in-person events for 25,000+ staff worldwide | Thousands of employees have completed Tetra Tech's Project Management Training program covering all phases of the project life cycle | Company offers accredited certification programs (IACET, APMG International, ANSI) and runs IP3 (Institute for Public-Private Partnerships), a Tetra Tech company providing PPP certification training</t>
+          <t>Uses structured mentoring relationships pairing employees with experienced staff to build skills for current and future roles | Provides financial support for external conferences, education, and training courses that benefit both employee and company | Funds a family scholarship program (MDU Resources Foundation) supporting employees' children/spouses in college or vocational education, suggesting a broader culture of investment in learning</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Tetra Tech FY2025 10-K Human Capital section + tetratech.com Learning and Development pages</t>
+          <t>MDU Resources careers site and MDU Resources Foundation scholarship program materials</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Arcadis U.S. Inc.</t>
+          <t>Sterling Construction</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1553,26 +1538,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C38" s="1" t="inlineStr">
-        <is>
-          <t>https://www.arcadis.com/</t>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://www.strlco.com/</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/874238/000087423826000024/strl-20251231.htm</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Arcadis Energy Transition Academy targets training or recruiting 2,500+ 'Arcadian' energy experts by 2027, backed by an in-house online platform (ETA@Home) with curated technical modules | Citizen Development program is a 3-month upskilling track in data, cloud, security, AI, and software development that produced a 40% increase in tech proficiency within 90 days | Arcadis Talent Academy is a 6-month paid-job-track program combining real project experience with language and soft-skills training; company also partnered with Pluralsight Skills for digital-fluency upskilling</t>
+          <t>All project employees receive hazard-specific training, with new hires undergoing initial safety orientation plus structured follow-up training through their first 90 days | Daily safety briefings led by project foremen and regular walkthroughs by managers/supervisors/safety staff reinforce continuous field-level training | Given ~3,000 employees and tight-labor-market hiring pressure, invests in structured onboarding and supervisory development to support retention, though no specific L&amp;D program names or figures were disclosed</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Arcadis.com newsroom, Arcadis 2024 Annual Integrated Report, Pluralsight case study</t>
+          <t>Sterling Infrastructure (Sterling Construction) FY2024 10-K human capital section</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Black &amp; Veatch</t>
+          <t>Dycom Industries</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1580,26 +1570,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C39" s="1" t="inlineStr">
-        <is>
-          <t>https://www.bv.com/</t>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://www.dycomind.com/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/67215/000006721526000008/dy-20260131.htm</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Black &amp; Veatch offers tuition assistance for full-time employee-owners, rated 4.0/5 by employees on Glassdoor for this benefit | ENT Accelerator Program is a full-time paid entry-level training track where trainees start earning pay and benefits on day one of class | As an employee-owned firm, the company bundles professional development with 401(k) match, professional-society support, and wellbeing programs as part of its 'people first' Total Rewards approach</t>
+          <t>Announced (Mar 2026) plans to build a flagship digital infrastructure workforce training center on a 49-acre campus in Monroe/Walton County, GA, opening mid-2027, with a simulated town for hands-on fiber deployment and a mock mission-critical facility for electrical systems training | This centralized hub complements Dycom's existing network of regional and field training centers, delivering immersive multi-week programs across its ~19,556-employee workforce | 10-K states employees receive training in specialized technical skills required to operate the business, plus mandatory Code of Conduct training and job-specific safety training</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Glassdoor Black &amp; Veatch benefits page, bv.com Early Careers/ENT Accelerator Program page</t>
+          <t>Dycom FY2026 10-K (SEC EDGAR) + GlobeNewswire Mar 2026 training center announcement</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CH2M</t>
+          <t>MYR Group</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1607,26 +1602,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C40" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ch2m.com/</t>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.myrgroup.com/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/700923/000070092326000007/myrg-20251231.htm</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>CH2M HILL no longer exists as a standalone company â€” Jacobs Engineering completed its acquisition on December 15, 2017 for ~$1.8B cash plus ~$1.4B of Jacobs stock, fully absorbing CH2M's workforce and operations | any legacy CH2M training programs (e.g., project management and technical certification tracks) were folded into Jacobs' own learning infrastructure post-merger | successor Jacobs Engineering runs enterprise-wide learning and leadership-development programs, including project-management and technical certification support</t>
+          <t>10-K names 'employee recruitment, training and development' as a core pillar of its human capital management strategy across ~9,000 employees (7,200 craft), most represented by IBEW | Subsidiary Harlan Electric Company runs the PLANT pre-apprenticeship program with Detroit's Public Lighting Authority and IBEW Local 17, training participants in OSHA 10, CPR/First Aid, and CDL before entering the NECA-IBEW Joint Apprenticeship Training Center pipeline | Craft workforce training is delivered largely through union apprenticeship channels (IBEW/NECA) rather than a standalone corporate university</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>SEC EDGAR Jacobs Engineering S-4/10-Q filings on the 2017 CH2M acquisition</t>
+          <t>MYR Group FY2025 10-K (SEC) + MYR Group newsroom (PLANT program, Aug 2024)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Burns &amp; McDonnell</t>
+          <t>Argan Inc.</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1634,26 +1634,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C41" s="1" t="inlineStr">
-        <is>
-          <t>https://www.burnsmcd.com/</t>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://www.arganinc.com/</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/100591/000110465926035216/agx-20260131x10k.htm</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Burns &amp; McDonnell delivers roughly 2,500 in-house company-led development classes per year spanning technical, computer, safety, and professional-development topics, taught online, in-person, and on-demand | Tuition reimbursement covers up to the IRS non-taxable limit annually for Bachelor's study and up to $10,000/year for Master's study, available to full-time employee-owners after 6 months of service | Employee-owners can earn Professional Development Hours (PDH) from completed courses, and the company pays professional/technical society membership dues plus offers career-counseling through its Professional Development Department</t>
+          <t>FY2026 10-K explicitly lists 'training and professional development initiatives' among its core employee-retention levers, across 1,409 employees | Industrial segment 10-K notes the company 'maintains training and safety programs designed to support workforce development' for its craft and project-leadership workforce | Subsidiary Gemma Power Systems (EPC arm) emphasizes hands-on training and mentorship for entry-level hires plus a strong safety-training culture</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>burnsmcd.com Training &amp; Development careers page; Glassdoor Burns &amp; McDonnell Tuition Assistance benefit page</t>
+          <t>Argan Inc FY2026 10-K (SEC EDGAR) + Gemma Power Systems careers page</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>HNTB Corporation</t>
+          <t>Comfort Systems USA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1661,26 +1666,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C42" s="1" t="inlineStr">
-        <is>
-          <t>https://www.hntb.com/</t>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://www.comfortsystemsusa.com/</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1035983/000110465926017530/fix-20251231x10k.htm</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Formal mentorship program pairs mentors and mentees for professional growth, plus tuition reimbursement/financial assistance for continuing education | HNTB Fellows Program recognizes top technical leadership, mentoring, and consulting achievement company-wide | Learning &amp; Development team manages training via Workday Learning, offering leadership courses, workshops, webinars, and structured onboarding for new hires and interns</t>
+          <t>10-K states the company provides 'numerous training programs for management, sales, and leadership, as well as on-the-job training, technical training, and apprenticeship programs' across ~22,700 employees | Offers 4-year apprenticeships in Plumbing, Sheet Metal, Electrical, and HVAC (NCCER/DOL-accredited), combining ~2,000 paid on-the-job hours with a minimum 144 classroom hours/year | Runs the Comfort Systems USA Technician Academy, an online technical-training platform with 1,500+ hours of content, plus local subsidiary academies and tuition reimbursement</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>HNTB corporate site, careers/FAQ pages</t>
+          <t>Comfort Systems USA FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Toll Brothers</t>
+          <t>KBR Inc.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1688,31 +1698,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C43" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tollbrothers.com/</t>
-        </is>
-      </c>
-      <c r="D43" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/794170/000079417025000112/tol-20251031.htm</t>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.kbr.com/</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1357615/000135761526000051/kbr-20260102.htm</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FY2025 10-K confirms mandatory annual training for all employees on preventing/reporting workplace discrimination as part of code of conduct | Company (approx. 4,900 full-time employees) states it focuses significant resources on attracting, developing, and retaining talented staff, monitored via engagement/satisfaction surveys | Sustainability reporting references leadership development, diversity training, and mentorship programs, though specific training-hour metrics are not publicly broken out</t>
+          <t>Offers Skillsoft Percipio learning platform with 50,000+ resources (videos, digital books, live Leadercasts, boot camps) available company-wide | Runs a Front-Line Leader (FLL) Program covering emotional awareness, communication, business acumen, and coaching skills for people managers | Provides an Education Reimbursement Program covering courses/certifications tied to role or promotion path, across ~36,000 employees in 28+ countries</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Toll Brothers FY2025 10-K (SEC EDGAR) human capital section + tollbrothers.com/sustainability</t>
+          <t>KBR FY2025/2026 10-K Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Quanta Services</t>
+          <t>Beazer Homes USA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1720,31 +1730,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C44" s="1" t="inlineStr">
-        <is>
-          <t>https://www.quantaservices.com/</t>
-        </is>
-      </c>
-      <c r="D44" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1050915/000105091526000006/pwr-20251231.htm</t>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.beazer.com/</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/915840/000091584025000075/bzh-20250930.htm</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Owns and operates Northwest Lineman College, a postsecondary institution specializing in pre-apprenticeship, apprenticeship, and specialized utility task training for electric workers | Operating companies run DOL-approved apprenticeship programs and participate in IBEW/NECA Apprenticeship Program and other union-sponsored craft training | Maintains strategic partnerships with universities, the military, and unions specifically to build and train its skilled-craft and engineering workforce</t>
+          <t>Runs construction 'Boot Camp' training programs specifically for new construction superintendents | Operates a dedicated sales training course teaching best practices, reinforced via national sales conferences and local training classes across markets | Workforce of ~1,158 employees with company-stated focus on comprehensive training/development programs plus safety and wellness training</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Quanta Services 10-K (FY2025, SEC EDGAR) human capital/workforce development disclosures</t>
+          <t>Beazer Homes FY2024/2025 10-K Human Capital disclosures</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Emerson Electric</t>
+          <t>M.D.C. Holdings</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1752,31 +1762,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C45" s="1" t="inlineStr">
-        <is>
-          <t>https://www.emerson.com/</t>
-        </is>
-      </c>
-      <c r="D45" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/32604/000003260425000087/emr-20250930.htm</t>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://www.richmondamerican.com/</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=MDC</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Runs global training and development programs explicitly aimed at building employees' leadership and professional skills, including intensive programs for both new and established leaders | Partners with educational institutions and nonprofit organizations to prepare current and future workers with needed skills | Approximately 73,000 employees company-wide (FY2024 count) supported by ongoing workplace-modernization and talent-development initiatives</t>
+          <t>Offers structured onboarding and job-specific training for sales, construction, and management roles similar to peer homebuilders, likely including online learning modules given a modest ~1,760-employee headcount | Uses job shadowing and mentoring as core development methods per 10-K human capital language | As a mid-size homebuilder, decision-making on formal L&amp;D vendors is probably centralized at HQ</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Emerson Electric FY2025 10-K (SEC EDGAR) human capital section + emerson.com/careers</t>
+          <t>MDC Holdings FY2023 10-K Human Capital Resources section â€” acquired by Sekisui House in 2024, no current standalone disclosures</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Jacobs Engineering</t>
+          <t>Hovnanian Enterprises</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1784,31 +1794,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C46" s="1" t="inlineStr">
-        <is>
-          <t>https://www.jacobs.com/</t>
-        </is>
-      </c>
-      <c r="D46" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/52988/000162828025053316/jec-20250926.htm</t>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.khov.com/</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/357294/000175392625001938/hov-20251031.htm</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Launched "Jacobs University" in fiscal 2025 as a global learning and development hub with four dedicated schools (more planned) and nearly 30,000 training programs, built in response to employee feedback for more AI/digital-skills training | Offers 32,000+ training programs through its e3 Learning platform tied to the "e3: engage. excel. elevate." employee experience framework | No explicit PMP/project-management certification program disclosed in the 10-K, but broad, high-volume internal learning infrastructure signals strong receptivity to external certification partnerships</t>
+          <t>Runs an Accelerated Leadership Development Program (ALDP) that mentors internal and external candidates for growth and succession planning, with active outreach to women and diverse candidates | Requires annual diversity &amp; inclusion training for all associates, with expanded D&amp;I training mandated for leadership-level staff | Training Department regularly conducts structured classes in sales, construction, administration, and managerial skills across ~1,878 full-time associates</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Jacobs Solutions FY2025 10-K (SEC EDGAR) human capital section</t>
+          <t>Hovnanian Enterprises FY2024 10-K Human Capital section</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MasTec</t>
+          <t>Taylor Morrison</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1816,31 +1826,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C47" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mastec.com/</t>
-        </is>
-      </c>
-      <c r="D47" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/15615/000001561526000020/mtz-20251231.htm</t>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://www.taylormorrison.com/</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1562476/000162828026009030/tmhc-20251231.htm</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Provides regular safety and skill-level training including safety leadership training for front-line leaders, OSHA construction outreach training, and operator qualification/electric worker training | Runs ongoing internally-developed educational programs combining classroom and field training to build technical and management skills | ~36,000 employees as of Dec 2025, with training/career development framed as a core retention and attraction strategy under its 'Zero Harm' safety culture</t>
+          <t>Provides tuition reimbursement for job-related coursework/books plus a college partnership letting full-time team members complete undergrad/graduate degrees | Runs the Voyager program, a dedicated pathway helping military veterans and skilled trade professionals transition into homebuilding careers | Offers ongoing leadership training and networking programs as part of its professional development track</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>MasTec FY2025 10-K (SEC EDGAR, mtz-20251231.htm) human capital section</t>
+          <t>Taylor Morrison FY2023 10-K Human Capital section + careers.taylormorrison.com</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Primoris Services</t>
+          <t>William Lyon Homes</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1848,31 +1858,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C48" s="1" t="inlineStr">
-        <is>
-          <t>https://www.prim.com/</t>
-        </is>
-      </c>
-      <c r="D48" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1361538/000110465926018677/prim-20251231x10k.htm</t>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.lyonhomes.com/</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Runs five-tier leadership development curriculum (Foreman Foundations, Extreme Ownership, Hunt for Leadership Success, Next Level Leadership, The Leadership Experience) progressing crew members to strategic leaders | Operates company-owned training facilities, including sites that train electric apprentices through to journeyman status | Provides project management training alongside on- and off-site skills training as part of its 'skilled labor advantage' strategy</t>
+          <t>William Lyon Homes was acquired by Taylor Morrison in a $2.4B deal that closed Feb 6, 2020, and no longer files independently, so no current standalone training disclosures exist | legacy training programs were folded into Taylor Morrison's onboarding and L&amp;D infrastructure post-merger | any pre-2020 training initiatives are no longer tracked as a distinct entity</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Primoris Services FY2024/2025 10-K human capital disclosures (SEC EDGAR)</t>
+          <t>SEC EDGAR Form 425 / Taylor Morrison-William Lyon merger coverage (Feb 2020)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MDU Resources</t>
+          <t>Century Communities</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1880,31 +1885,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C49" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mdu.com/</t>
-        </is>
-      </c>
-      <c r="D49" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/67716/000006771626000014/mdu-20251231.htm</t>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://www.centurycommunities.com/</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1576940/000157694026000005/ccs-20251231x10k.htm</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Uses structured mentoring relationships pairing employees with experienced staff to build skills for current and future roles | Provides financial support for external conferences, education, and training courses that benefit both employee and company | Funds a family scholarship program (MDU Resources Foundation) supporting employees' children/spouses in college or vocational education, suggesting a broader culture of investment in learning</t>
+          <t>Runs an internal 'Century University' offering a learning management system with training videos/quizzes on construction, customer relations, purchasing, land development and safety | Provides field training for construction and sales staff led by internal and external subject-matter experts, plus periodic leadership seminars for executives | Maintains a formal 'Commitment to Training and Professional Development' policy covering company policy, anti-harassment, anti-discrimination and sales training</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>MDU Resources careers site and MDU Resources Foundation scholarship program materials</t>
+          <t>Century Communities FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Granite Construction</t>
+          <t>Green Brick Partners</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1912,31 +1917,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C50" s="1" t="inlineStr">
-        <is>
-          <t>https://www.graniteconstruction.com/</t>
-        </is>
-      </c>
-      <c r="D50" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/861459/000086145926000004/gva-20251231.htm</t>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.greenbrickpartners.com/</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1373670/000162828026011798/grbk-20251231.htm</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Employees completed over 35,000 training courses in 2025 combining on-the-job learning with in-person and online coursework | More than 200 employees graduated from Granite's multi-level leadership development program in 2025, spanning emerging to senior leaders | Managerial/supervisory staff average 12 years tenure, attributed to sustained investment in talent development and succession planning</t>
+          <t>Sales force trained through 'comprehensive training programs' paired with advanced digital tools, per FY2025 10-K human capital section | Mandatory annual cybersecurity/education-and-awareness training required for all personnel, with bi-weekly phishing-campaign testing | Employees who fail phishing tests are automatically re-enrolled in cybersecurity awareness training</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Granite Construction FY2025 10-K (SEC EDGAR, gva-20251231.htm) human capital section</t>
+          <t>Green Brick Partners FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Sterling Construction</t>
+          <t>LGI Homes</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1944,31 +1949,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C51" s="1" t="inlineStr">
-        <is>
-          <t>https://www.strlco.com/</t>
-        </is>
-      </c>
-      <c r="D51" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/874238/000087423826000024/strl-20251231.htm</t>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.lgihomes.com/</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1580670/000158067026000019/lgih-20251231.htm</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>All project employees receive hazard-specific training, with new hires undergoing initial safety orientation plus structured follow-up training through their first 90 days | Daily safety briefings led by project foremen and regular walkthroughs by managers/supervisors/safety staff reinforce continuous field-level training | Given ~3,000 employees and tight-labor-market hiring pressure, invests in structured onboarding and supervisory development to support retention, though no specific L&amp;D program names or figures were disclosed</t>
+          <t>Runs a structured 100-day sales training program: 30 days of intensive in-house instruction on proprietary selling strategies followed by field training at the local division | Holds ongoing weekly training sessions at every information center plus quarterly regional training events for sales personnel | Routine employee cyber/information-security training required company-wide</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Sterling Infrastructure (Sterling Construction) FY2024 10-K human capital section</t>
+          <t>LGI Homes FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Dycom Industries</t>
+          <t>M/I Homes</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1976,31 +1981,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C52" s="1" t="inlineStr">
-        <is>
-          <t>https://www.dycomind.com/</t>
-        </is>
-      </c>
-      <c r="D52" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/67215/000006721526000008/dy-20260131.htm</t>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.mihomes.com/</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/799292/000079929226000006/mho-20251231.htm</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Announced (Mar 2026) plans to build a flagship digital infrastructure workforce training center on a 49-acre campus in Monroe/Walton County, GA, opening mid-2027, with a simulated town for hands-on fiber deployment and a mock mission-critical facility for electrical systems training | This centralized hub complements Dycom's existing network of regional and field training centers, delivering immersive multi-week programs across its ~19,556-employee workforce | 10-K states employees receive training in specialized technical skills required to operate the business, plus mandatory Code of Conduct training and job-specific safety training</t>
+          <t>Operating divisions assign role-specific training aligned to each employee's responsibilities and career aspirations | Mandatory company-wide training sessions cover workplace safety, ethics, cybersecurity and anti-harassment for all employees | All employees must complete biannual security-awareness training on data protection and phishing prevention</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Dycom FY2026 10-K (SEC EDGAR) + GlobeNewswire Mar 2026 training center announcement</t>
+          <t>M/I Homes FY2025 10-K (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MYR Group</t>
+          <t>New Home Company</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2008,31 +2013,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C53" s="1" t="inlineStr">
-        <is>
-          <t>https://www.myrgroup.com/</t>
-        </is>
-      </c>
-      <c r="D53" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/700923/000070092326000007/myrg-20251231.htm</t>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://www.nwhm.com/</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=NWHM</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>10-K names 'employee recruitment, training and development' as a core pillar of its human capital management strategy across ~9,000 employees (7,200 craft), most represented by IBEW | Subsidiary Harlan Electric Company runs the PLANT pre-apprenticeship program with Detroit's Public Lighting Authority and IBEW Local 17, training participants in OSHA 10, CPR/First Aid, and CDL before entering the NECA-IBEW Joint Apprenticeship Training Center pipeline | Craft workforce training is delivered largely through union apprenticeship channels (IBEW/NECA) rather than a standalone corporate university</t>
+          <t>New Home Company was taken private by Apollo Global Management in a deal completed Sept 8, 2021, and no longer publicly discloses training programs | as an Apollo portfolio homebuilder, sales and safety training programs were likely standardized/absorbed rather than published independently | any CA/AZ/CO regional training initiatives from its public era are no longer separately reported</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>MYR Group FY2025 10-K (SEC) + MYR Group newsroom (PLANT program, Aug 2024)</t>
+          <t>Apollo Global Management press release (Sept 2021) / SEC EDGAR 8-K filings</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Argan Inc.</t>
+          <t>Vanir Construction Management</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2040,31 +2045,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C54" s="1" t="inlineStr">
-        <is>
-          <t>https://www.arganinc.com/</t>
-        </is>
-      </c>
-      <c r="D54" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/100591/000110465926035216/agx-20260131x10k.htm</t>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.vanir.com/</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>FY2026 10-K explicitly lists 'training and professional development initiatives' among its core employee-retention levers, across 1,409 employees | Industrial segment 10-K notes the company 'maintains training and safety programs designed to support workforce development' for its craft and project-leadership workforce | Subsidiary Gemma Power Systems (EPC arm) emphasizes hands-on training and mentorship for entry-level hires plus a strong safety-training culture</t>
+          <t>Offers 'Vanir University,' an internal online course catalog for staff professional development plus industry-association memberships | Pays for CMAA training and Certified Construction Manager (CCM) exam prep/review for staff pursuing certification | Developing a formal mentorship program pairing new hires with experienced mentors outside their direct reporting line</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Argan Inc FY2026 10-K (SEC EDGAR) + Gemma Power Systems careers page</t>
+          <t>Vanir company careers/about-us pages</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Comfort Systems USA</t>
+          <t>Swinerton</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2072,31 +2072,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C55" s="1" t="inlineStr">
-        <is>
-          <t>https://www.comfortsystemsusa.com/</t>
-        </is>
-      </c>
-      <c r="D55" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1035983/000110465926017530/fix-20251231x10k.htm</t>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://www.swinerton.com/</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>10-K states the company provides 'numerous training programs for management, sales, and leadership, as well as on-the-job training, technical training, and apprenticeship programs' across ~22,700 employees | Offers 4-year apprenticeships in Plumbing, Sheet Metal, Electrical, and HVAC (NCCER/DOL-accredited), combining ~2,000 paid on-the-job hours with a minimum 144 classroom hours/year | Runs the Comfort Systems USA Technician Academy, an online technical-training platform with 1,500+ hours of content, plus local subsidiary academies and tuition reimbursement</t>
+          <t>Runs 'LeaderBuilder,' an intensive leadership-development series for managers on organizational, communication and motivational skills | 'Better Builders' program gives project engineers field experience and on-the-job training in core construction techniques | 100% employee-owned (ESOP) structure paired with 'career blueprints' mapping the skills/training needed at each leadership level, plus a separate 'Craft Leader' training track for field craft staff</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Comfort Systems USA FY2025 10-K (SEC EDGAR)</t>
+          <t>Swinerton corporate site (careers, culture, talent-pipeline pages)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Tutor Perini</t>
+          <t>The Weitz Company</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2104,31 +2099,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C56" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tutorperini.com/</t>
-        </is>
-      </c>
-      <c r="D56" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/77543/000007754326000028/tpc-20251231.htm</t>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://www.weitz.com/</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>10-K frames training/retention as a core strategic pillar ('Talent Recruitment, Training and Retention') across ~7,400 employees, delivered via management information systems, on-the-job training, and educational seminars | Places particular emphasis on training staff in project estimating, project management, and project cost control, building a pipeline of long-term successors to current project leaders | Runs an active college recruitment program pulling from construction management, civil, mechanical, and electrical engineering programs nationwide</t>
+          <t>Launched 'Weitz University,' an internally facilitated educational program aimed at expanding contracting opportunities and reducing barriers for small/diverse businesses | Every employee is promised a defined career path supported by structured training and development opportunities | Annual mandatory inclusion training required for all employees</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Tutor Perini FY2025 10-K (SEC EDGAR) + Tutor Perini careers/college recruitment pages</t>
+          <t>Weitz Company careers site</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>KBR Inc.</t>
+          <t>PCL Construction</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2136,31 +2126,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C57" s="1" t="inlineStr">
-        <is>
-          <t>https://www.kbr.com/</t>
-        </is>
-      </c>
-      <c r="D57" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1357615/000135761526000051/kbr-20260102.htm</t>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://www.pcl.com/</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Offers Skillsoft Percipio learning platform with 50,000+ resources (videos, digital books, live Leadercasts, boot camps) available company-wide | Runs a Front-Line Leader (FLL) Program covering emotional awareness, communication, business acumen, and coaching skills for people managers | Provides an Education Reimbursement Program covering courses/certifications tied to role or promotion path, across ~36,000 employees in 28+ countries</t>
+          <t>In-house 'PCL College of Construction' has delivered 2,000+ custom courses over 25+ years spanning technical, leadership and behavioral training | 'E3 Leadership Certification Program' has produced 1,000+ graduates since launching in 2017, open to employees at any level | Reimburses up to $1,000/year per employee for off-site work-related education, plus conference and certification expenses; also runs a formal cross-department mentorship program</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>KBR FY2025/2026 10-K Human Capital section</t>
+          <t>PCL Construction insights pages and careers FAQ</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Beazer Homes USA</t>
+          <t>Archer Western Construction</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2168,31 +2153,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C58" s="1" t="inlineStr">
-        <is>
-          <t>https://www.beazer.com/</t>
-        </is>
-      </c>
-      <c r="D58" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/915840/000091584025000075/bzh-20250930.htm</t>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://www.walshgroup.com/archer-western.html</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Runs construction 'Boot Camp' training programs specifically for new construction superintendents | Operates a dedicated sales training course teaching best practices, reinforced via national sales conferences and local training classes across markets | Workforce of ~1,158 employees with company-stated focus on comprehensive training/development programs plus safety and wellness training</t>
+          <t>as part of the family-owned Walsh Group, Archer Western follows shared safety-first training culture ('No One Gets Hurt') applied across its roughly 8,000 combined employees | entry-level and skilled-craft employees get structured industry training tied to career advancement, per Walsh Group careers messaging | dedicated safety/training management roles exist within the shared Walsh Group organizational structure</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Beazer Homes FY2024/2025 10-K Human Capital disclosures</t>
+          <t>Walsh Group corporate/careers and safety pages</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>M.D.C. Holdings</t>
+          <t>Clark Construction Group</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2200,31 +2180,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C59" s="1" t="inlineStr">
-        <is>
-          <t>https://www.richmondamerican.com/</t>
-        </is>
-      </c>
-      <c r="D59" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=MDC</t>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://www.clarkconstruction.com/</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Offers structured onboarding and job-specific training for sales, construction, and management roles similar to peer homebuilders, likely including online learning modules given a modest ~1,760-employee headcount | Uses job shadowing and mentoring as core development methods per 10-K human capital language | As a mid-size homebuilder, decision-making on formal L&amp;D vendors is probably centralized at HQ</t>
+          <t>In-house learning academy 'CCU' offers 100+ classes for employees at every career stage, supplemented by on-demand LinkedIn Learning access | 'Bootcamp' program prepares engineers to transition into management, while the Field Development Group (FDG) grooms candidates for superintendent roles | Offers tuition reimbursement for formal courses of study and runs a robust seasonal internship program with structured mentorship</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>MDC Holdings FY2023 10-K Human Capital Resources section â€” acquired by Sekisui House in 2024, no current standalone disclosures</t>
+          <t>Clark Construction careers site</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Hovnanian Enterprises</t>
+          <t>Haskell</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2232,31 +2207,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C60" s="1" t="inlineStr">
-        <is>
-          <t>https://www.khov.com/</t>
-        </is>
-      </c>
-      <c r="D60" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/357294/000175392625001938/hov-20251031.htm</t>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://www.haskell.com/</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Runs an Accelerated Leadership Development Program (ALDP) that mentors internal and external candidates for growth and succession planning, with active outreach to women and diverse candidates | Requires annual diversity &amp; inclusion training for all associates, with expanded D&amp;I training mandated for leadership-level staff | Training Department regularly conducts structured classes in sales, construction, administration, and managerial skills across ~1,878 full-time associates</t>
+          <t>Ranked No. 1 in Training Magazine's APEX Awards for leading training organizations, reflecting major investment across its 2,300+ team members | Team members logged over 104,000 training hours in 2022, a 67% year-over-year increase, largely through 'Haskell University' LMS | Permanent Craft Employee (PCE) program combined with the Field Technical Training (FTT) curriculum helps tradespeople earn professional certifications; leadership development runs through the EPIC coaching program</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Hovnanian Enterprises FY2024 10-K Human Capital section</t>
+          <t>Haskell company insights pages and Training Magazine APEX Awards coverage</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Taylor Morrison</t>
+          <t>Mortenson Construction</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2264,31 +2234,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C61" s="1" t="inlineStr">
-        <is>
-          <t>https://www.taylormorrison.com/</t>
-        </is>
-      </c>
-      <c r="D61" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1562476/000162828026009030/tmhc-20251231.htm</t>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://www.mortenson.com/</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Provides tuition reimbursement for job-related coursework/books plus a college partnership letting full-time team members complete undergrad/graduate degrees | Runs the Voyager program, a dedicated pathway helping military veterans and skilled trade professionals transition into homebuilding careers | Offers ongoing leadership training and networking programs as part of its professional development track</t>
+          <t>'Pathways Leadership Development Program' creates structured leadership-growth opportunities; 'LeadBLU' pairs leadership development with inclusion training | Piloted a two-day immersive hybrid skills-training experience for Project Managers and Superintendents | Launched its first-ever NCCER-accredited carpenter apprenticeship class (Mortenson Phoenix) as part of broader workforce-development efforts</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Taylor Morrison FY2023 10-K Human Capital section + careers.taylormorrison.com</t>
+          <t>Mortenson news/insights pages</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Tri Pointe Homes</t>
+          <t>Sundt Construction</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2296,31 +2261,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C62" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tripointehomes.com/</t>
-        </is>
-      </c>
-      <c r="D62" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=TPH</t>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://www.sundt.com/</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Offers structured sales-rep development including day-one access to a 'Blueprint' leadership and learning program | Tuition reimbursement provided as part of employee benefits | Leadership training and internal promotion paths are formal growth tracks</t>
+          <t>100% employee-owned; Talent Development Program centers on the Sundt Training Center and Center for Craft Excellence, expanded via the G. Michael Hoover KAPBCS Training Center opened in 2023 | Runs multiple DOL-approved NCCER apprenticeship tracks (heavy equipment operation, electrician, pipefitter, ironworker, craft laborer) with pay and benefits during training | 'LEAP' (Leadership Excellence Accelerates Performance) is a nationally recognized program preparing employee-owners for mid-level and senior leadership roles</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Tri Pointe Homes careers site / employer profiles</t>
+          <t>Sundt Construction training/careers pages</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Meritage Homes</t>
+          <t>layton construction</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2328,31 +2288,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C63" s="1" t="inlineStr">
-        <is>
-          <t>https://www.meritagehomes.com/</t>
-        </is>
-      </c>
-      <c r="D63" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/833079/000083307926000010/mth-20251231.htm</t>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://www.laytonconstruction.com/</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>FY2025 10-K highlights tuition reimbursement as a standing employee benefit | Mandatory ongoing information-security/cybersecurity training required company-wide, including monthly phishing simulations | Workforce is 42% female and 58% minority as of Dec 31, 2025, per human capital disclosures</t>
+          <t>Company states it "invests significantly in employee development because excellence drives our industry" and promotes based on performance rather than tenure/seniority | Runs a structured internship program recruiting university students nationwide for hands-on, mentored experience across technology, marketing, finance and operations | offers on-the-job mentoring and safety/technical training typical of large regional GCs, though no named academy or PMP/PMI partnership is publicly documented</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Meritage Homes FY2025 10-K (SEC EDGAR)</t>
+          <t>laytonconstruction.com/careers/</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>William Lyon Homes</t>
+          <t>Ryan Companies</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2360,26 +2315,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C64" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lyonhomes.com/</t>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://www.ryancompanies.com/</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>William Lyon Homes was acquired by Taylor Morrison in a $2.4B deal that closed Feb 6, 2020, and no longer files independently, so no current standalone training disclosures exist | legacy training programs were folded into Taylor Morrison's onboarding and L&amp;D infrastructure post-merger | any pre-2020 training initiatives are no longer tracked as a distinct entity</t>
+          <t>Formal Leadership Framework with named programs: NEO (2-day new-hire immersion), Manager Essentials (2.5-day new-manager training), Leading with Influence (multi-day senior leader program), and Team Excellence Program (1-day team workshop) | BUILd program grooms high-potential Assistant Superintendents for promotion and includes AGC Construction Supervision Fundamentals (CSF) certification upon completion | Four formal training tracks: Personal/Professional Development, Management/Leadership Development, Job Skill/Functional Training, and Safety/Quality/Scheduling Training</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>SEC EDGAR Form 425 / Taylor Morrison-William Lyon merger coverage (Feb 2020)</t>
+          <t>ryancompanies.com/careers/learning-development/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Century Communities</t>
+          <t>The Beck Group</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2387,31 +2342,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C65" s="1" t="inlineStr">
-        <is>
-          <t>https://www.centurycommunities.com/</t>
-        </is>
-      </c>
-      <c r="D65" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1576940/000157694026000005/ccs-20251231x10k.htm</t>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://www.beckgroup.com/</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Runs an internal 'Century University' offering a learning management system with training videos/quizzes on construction, customer relations, purchasing, land development and safety | Provides field training for construction and sales staff led by internal and external subject-matter experts, plus periodic leadership seminars for executives | Maintains a formal 'Commitment to Training and Professional Development' policy covering company policy, anti-harassment, anti-discrimination and sales training</t>
+          <t>Operates the Beck School of Construction (BSOC), a free 10-month training program (since 2019) for minority- and women-owned construction business leaders, now in Dallas, Fort Worth, Atlanta and Austin | Beck School of Construction has an OSHA safety alliance embedded in its curriculum and has helped graduates win over $15 million in project work | Careers page references company-wide learning/leadership and internship programs</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Century Communities FY2025 10-K (SEC EDGAR)</t>
+          <t>beckgroup.com/careers/ and beckgroup.com/the-beck-school-of-construction/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Green Brick Partners</t>
+          <t>Barton Malow Company</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2419,31 +2369,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C66" s="1" t="inlineStr">
-        <is>
-          <t>https://www.greenbrickpartners.com/</t>
-        </is>
-      </c>
-      <c r="D66" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1373670/000162828026011798/grbk-20251231.htm</t>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://www.bartonmalow.com/</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Sales force trained through 'comprehensive training programs' paired with advanced digital tools, per FY2025 10-K human capital section | Mandatory annual cybersecurity/education-and-awareness training required for all personnel, with bi-weekly phishing-campaign testing | Employees who fail phishing tests are automatically re-enrolled in cybersecurity awareness training</t>
+          <t>Runs the Barton Malow Boot Camp (launched 2016), a paid 120-hour, 6-week pre-apprenticeship program for residents aged 18-24 covering OSHA, financial literacy, soft skills and hands-on trades training with a mentor; 150+ graduates | Built dedicated hands-on Autodesk Construction Cloud training labs and ran recurring in-person/virtual training for roughly 3,500 employees across 14 offices | Won AGC Cornerstone Award (2024, 2026) and AGC Community Award (2020) for workforce development</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Green Brick Partners FY2025 10-K (SEC EDGAR)</t>
+          <t>bartonmalow.com/about-us/diversity-equity-inclusion/workforce-development/</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LGI Homes</t>
+          <t>McCarthy Building Companies</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2451,31 +2396,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C67" s="1" t="inlineStr">
-        <is>
-          <t>https://www.lgihomes.com/</t>
-        </is>
-      </c>
-      <c r="D67" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1580670/000158067026000019/lgih-20251231.htm</t>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://www.mccarthy.com/</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Runs a structured 100-day sales training program: 30 days of intensive in-house instruction on proprietary selling strategies followed by field training at the local division | Holds ongoing weekly training sessions at every information center plus quarterly regional training events for sales personnel | Routine employee cyber/information-security training required company-wide</t>
+          <t>Named learning program "McCarthy BUILD U" blends orientation, a personal curriculum, virtual and instructor-led classroom training, action learning, and peer-to-peer mentoring, plus tuition reimbursement | Purchased a 12-acre former hotel/convention site in Tempe, AZ to build a dedicated leadership-and-culture development campus, alongside its Innovation and Craft Workforce Center | First construction company inducted into Training Magazine's Training Top-10 Hall of Fame; 100% employee-owned since 2002</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>LGI Homes FY2025 10-K (SEC EDGAR)</t>
+          <t>mccarthy.com/careers/learning-development</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>M/I Homes</t>
+          <t>Holder Construction Company</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2483,31 +2423,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C68" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mihomes.com/</t>
-        </is>
-      </c>
-      <c r="D68" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/799292/000079929226000006/mho-20251231.htm</t>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://www.holderconstruction.com/</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Operating divisions assign role-specific training aligned to each employee's responsibilities and career aspirations | Mandatory company-wide training sessions cover workplace safety, ethics, cybersecurity and anti-harassment for all employees | All employees must complete biannual security-awareness training on data protection and phishing prevention</t>
+          <t>Runs HolderRISE, a paid high-school internship for ages 16-17 that rotates participants through safety, field supervision, MEP and quality-assurance roles | Offers a dedicated Career Paths &amp; Development track plus an Early Career Professionals program | Readiness programs for craft professionals combine structured training, mentorship, and defined career pathways</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>M/I Homes FY2025 10-K (SEC EDGAR)</t>
+          <t>holderconstruction.com careers/development pages</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>New Home Company</t>
+          <t>Structure Tone</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2515,31 +2450,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C69" s="1" t="inlineStr">
-        <is>
-          <t>https://www.nwhm.com/</t>
-        </is>
-      </c>
-      <c r="D69" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?CIK=NWHM</t>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://www.structuretone.com/</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>New Home Company was taken private by Apollo Global Management in a deal completed Sept 8, 2021, and no longer publicly discloses training programs | as an Apollo portfolio homebuilder, sales and safety training programs were likely standardized/absorbed rather than published independently | any CA/AZ/CO regional training initiatives from its public era are no longer separately reported</t>
+          <t>Runs an RPE Program that places entry-level architecture, civil engineering, construction management and interior design graduates into a structured, mentor-guided rotational experience | Participates in the ACE Mentor Program of Greater New York, pairing staff mentors with high-school student teams on real-world design/construction projects | Parent company STO Building Group provides tuition financial assistance plus a separate Women in Construction mentoring pilot</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Apollo Global Management press release (Sept 2021) / SEC EDGAR 8-K filings</t>
+          <t>stobuildinggroup.com (Structure Tone's parent, STO Building Group)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Vanir Construction Management</t>
+          <t>NOVA Engineering and Environmental</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2547,26 +2477,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C70" s="1" t="inlineStr">
-        <is>
-          <t>https://www.vanir.com/</t>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://www.novaenv.com/</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Offers 'Vanir University,' an internal online course catalog for staff professional development plus industry-association memberships | Pays for CMAA training and Certified Construction Manager (CCM) exam prep/review for staff pursuing certification | Developing a formal mentorship program pairing new hires with experienced mentors outside their direct reporting line</t>
+          <t>Certification pay bumps and bonuses tied to obtaining professional certifications, confirmed by multiple employee reviews | Employees are described as "mentored for the future" as part of a stated professional-development approach on the company careers page | Employee reviews (Glassdoor) indicate training/certification study materials are not centrally provided, requiring self-directed effort outside work hours</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Vanir company careers/about-us pages</t>
+          <t>usanova.com/careers and Glassdoor employee reviews</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Swinerton</t>
+          <t>STV Group</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2574,26 +2504,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C71" s="1" t="inlineStr">
-        <is>
-          <t>https://www.swinerton.com/</t>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://www.stv.com/</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Runs 'LeaderBuilder,' an intensive leadership-development series for managers on organizational, communication and motivational skills | 'Better Builders' program gives project engineers field experience and on-the-job training in core construction techniques | 100% employee-owned (ESOP) structure paired with 'career blueprints' mapping the skills/training needed at each leadership level, plus a separate 'Craft Leader' training track for field craft staff</t>
+          <t>Offers a formal tuition reimbursement program alongside professional development seminars and online education initiatives | Provides technical training paired with dedicated mentors as part of its career-development approach | Supports 10+ employee-led community/network groups (e.g., Women's Network, Rising Professionals, Veterans &amp; Military) that also serve as professional-development channels</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Swinerton corporate site (careers, culture, talent-pipeline pages)</t>
+          <t>stvinc.com careers pages</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>The Weitz Company</t>
+          <t>Gannett Fleming</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2601,26 +2531,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C72" s="1" t="inlineStr">
-        <is>
-          <t>https://www.weitz.com/</t>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://www.gannettfleming.com/</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Launched 'Weitz University,' an internally facilitated educational program aimed at expanding contracting opportunities and reducing barriers for small/diverse businesses | Every employee is promised a defined career path supported by structured training and development opportunities | Annual mandatory inclusion training required for all employees</t>
+          <t>Runs a multi-tier instructor-led program ladder: PM Foundations, PM Academy, Project Principal Bootcamp, LEAD Manager Training, and Emerging Leaders | Provides a PMP Exam Preparation Program and FE/PE Exam Prep courses, plus tuition reimbursement and on-demand access to Percipio, LinkedIn Learning, Revit and Bentley training platforms | Runs a Connected Relationships Mentoring Program (fourth cycle, 4.5+/5 rating) plus an Internal Growth Opportunities internal-mobility program</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Weitz Company careers site</t>
+          <t>gftinc.com (Gannett Fleming) career-empowerment and learning-and-development pages</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>PCL Construction</t>
+          <t>WSP USA</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2628,26 +2558,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C73" s="1" t="inlineStr">
-        <is>
-          <t>https://www.pcl.com/</t>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://www.wsp.com/en-US</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>In-house 'PCL College of Construction' has delivered 2,000+ custom courses over 25+ years spanning technical, leadership and behavioral training | 'E3 Leadership Certification Program' has produced 1,000+ graduates since launching in 2017, open to employees at any level | Reimburses up to $1,000/year per employee for off-site work-related education, plus conference and certification expenses; also runs a formal cross-department mentorship program</t>
+          <t>Parent WSP Global's 2024 Global Sustainability Report cites 98.6% completion rate for Code of Conduct onboarding training across the workforce | WSP Learns platform gives all permanent employees global access to Inclusion &amp; Belonging training modules | WSP also runs REACH, an online training platform offering 24/7 self-directed learning plus enrollment in virtual and in-person sessions</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>PCL Construction insights pages and careers FAQ</t>
+          <t>WSP 2024 Global Sustainability Report; WSP careers/benefits pages</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Whiting-Turner Contracting Company</t>
+          <t>Atkins North America</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2655,26 +2585,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C74" s="1" t="inlineStr">
-        <is>
-          <t>https://www.whiting-turner.com/</t>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://www.atkinsglobal.com/en-US</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Offers tuition reimbursement up to $5,250/year for job-related coursework | Maintains a formal mentorship program pairing employees with peers and leaders for career development | Employee reviews and company messaging emphasize frequent training opportunities as part of career-goal support</t>
+          <t>AtkinsRealis (parent of Atkins North America) delivered classroom/webinar training to over 25,415 staff plus 468,309 online e-learning module completions, totaling almost 250,000 training hours | ESG-linked compensation ties 10% of the Annual Incentive Plan to metrics including Integrity, Health &amp; Safety, and Equality/Diversity &amp; Inclusion | Annual Integrated Report frames employee engagement and professional development as a core pillar of company strategy</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Whiting-Turner careers site</t>
+          <t>AtkinsRealis 2024 Annual Integrated Report / ESG disclosures</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>AstraZeneca's US Construction Partner, Jacobs</t>
+          <t>Michael Baker International</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2682,31 +2612,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C75" s="1" t="inlineStr">
-        <is>
-          <t>https://www.jacobs.com/</t>
-        </is>
-      </c>
-      <c r="D75" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/52988/000162828025053316/jec-20250926.htm</t>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://www.mbakerintl.com/</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Launched 'Jacobs University,' a global learning and development hub with four dedicated schools and near 30,000 available training programs, emphasizing AI and digital-skills upskilling | In fiscal 2025, over 97% of employees completed the mandatory annual 'Living Our Values' training module | Global graduate development program and local apprenticeships onboarded 1,300+ graduates, interns and apprentices in fiscal 2025</t>
+          <t>Runs a structured company-wide Mentorship Program pairing mentors and mentees for skill development and knowledge sharing | Internship program brings in more than 100 students annually for hands-on experience | Employee survey data shows 82% report being supported to advance their career and 72% report receiving adequate training when starting</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Jacobs Engineering Group FY2025 10-K (SEC EDGAR)</t>
+          <t>Michael Baker International careers site; Glassdoor employer profile</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Bechtel Group</t>
+          <t>Aptim</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2714,26 +2639,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C76" s="1" t="inlineStr">
-        <is>
-          <t>https://www.bechtel.com/</t>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://www.aptim.com/</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Runs 'Bechtel University,' offering thousands of instructor-led, virtual and mobile courses across leadership, technical, safety/ethics and language training | Four-week 'Construction Immersion' program accelerates onboarding for early-career construction professionals | 'Bechtel Field Leadership Assessment' and 'High-Performance Crews' program specifically develop front-line/field leaders</t>
+          <t>Offers tuition reimbursement for full-time salaried employees after one year of service, plus company-funded training, credentials, and certifications available to all employees on request | Provides every employee access to an online library of thousands of professional/personal development videos | Runs the THRIVE mentorship program; in 2023, 90% of professional employees completed required development-planning conversations with managers</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Bechtel corporate site (learning &amp; development page)</t>
+          <t>APTIM 2023 ESG Disclosures; APTIM careers page</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Archer Western Construction</t>
+          <t>CDM Smith</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2741,26 +2666,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C77" s="1" t="inlineStr">
-        <is>
-          <t>https://www.walshgroup.com/archer-western.html</t>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://www.cdm smith.com/</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>as part of the family-owned Walsh Group, Archer Western follows shared safety-first training culture ('No One Gets Hurt') applied across its roughly 8,000 combined employees | entry-level and skilled-craft employees get structured industry training tied to career advancement, per Walsh Group careers messaging | dedicated safety/training management roles exist within the shared Walsh Group organizational structure</t>
+          <t>Operates CDM Smith University, an IACET-accredited internal training institution founded nearly 30 years ago to advance technical skills and maintain professional certifications/registrations | Runs a formal Leadership Academy offering customizable development planning based on career stage | Also offers the Career Compass mentoring program, an Emerging Professionals Network, and a Reboot Re-Entry Program for employees returning from career breaks</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Walsh Group corporate/careers and safety pages</t>
+          <t>CDM Smith careers/career development pages</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Clark Construction Group</t>
+          <t>Louis Berger</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2768,26 +2693,26 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C78" s="1" t="inlineStr">
-        <is>
-          <t>https://www.clarkconstruction.com/</t>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://www.louisberger.com/</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>In-house learning academy 'CCU' offers 100+ classes for employees at every career stage, supplemented by on-demand LinkedIn Learning access | 'Bootcamp' program prepares engineers to transition into management, while the Field Development Group (FDG) grooms candidates for superintendent roles | Offers tuition reimbursement for formal courses of study and runs a robust seasonal internship program with structured mentorship</t>
+          <t>as a wholly absorbed WSP subsidiary since 2018, former Louis Berger staff would have transitioned to WSP's global learning management system and leadership development curriculum rather than retaining a standalone program | engineering/infrastructure staff would receive PE licensure support, continuing education credits, and technical certification reimbursement consistent with WSP's broader human capital practices | any legacy Louis Berger training identity or branding would have been phased out and folded into a WSP corporate L&amp;D platform post-acquisition</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Clark Construction careers site</t>
+          <t>Louis Berger acquired by WSP Global in 2018 (~$400M deal); no standalone disclosures exist post-acquisition</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Haskell</t>
+          <t>Parsons Corporation</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2795,26 +2720,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C79" s="1" t="inlineStr">
-        <is>
-          <t>https://www.haskell.com/</t>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://www.parsons.com/</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/275880/000119312526045495/psn-20251231.htm</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Ranked No. 1 in Training Magazine's APEX Awards for leading training organizations, reflecting major investment across its 2,300+ team members | Team members logged over 104,000 training hours in 2022, a 67% year-over-year increase, largely through 'Haskell University' LMS | Permanent Craft Employee (PCE) program combined with the Field Technical Training (FTT) curriculum helps tradespeople earn professional certifications; leadership development runs through the EPIC coaching program</t>
+          <t>Parsons Learning Series offers live, virtual one-hour courses monthly across topics for employees and managers, run at three time slots globally and recorded for later access | Engaged Leadership Program (ELP) is a 4-month cohort-based program building management/leadership skills, plus the Intentional Leadership Program (ILP), a facilitated 2-day curriculum for Director-level and above senior leaders | Fellows Program recognizes 50+ top technical experts; over 3,600 of ~21,000 employees hold advanced degrees/professional credentials</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Haskell company insights pages and Training Magazine APEX Awards coverage</t>
+          <t>Parsons Corporation FY2025 10-K, Human Capital Management section (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Mortenson Construction</t>
+          <t xml:space="preserve"> Tutor Perini Building Corp</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2822,26 +2752,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C80" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mortenson.com/</t>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://www.tutorperini.com/</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/77543/000007754326000028/tpc-20251231.htm</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>'Pathways Leadership Development Program' creates structured leadership-growth opportunities; 'LeadBLU' pairs leadership development with inclusion training | Piloted a two-day immersive hybrid skills-training experience for Project Managers and Superintendents | Launched its first-ever NCCER-accredited carpenter apprenticeship class (Mortenson Phoenix) as part of broader workforce-development efforts</t>
+          <t>Talent Recruitment, Training and Retention is named as a primary human capital goal, using management information systems, on-the-job training, and educational seminars, with heavy emphasis on project estimating, project management, and cost control training | Extensive safety training programs are mandatory, including an initial safety orientation for all new job-site hires and a required OSHA 30-hour training program | Company regularly hires construction management/engineering interns and recent graduates to build long-term successor project managers, across roughly 7,400 employees</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Mortenson news/insights pages</t>
+          <t>Tutor Perini Building Corp FY2025 10-K, Human Capital Resources section (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Sundt Construction</t>
+          <t>Ameresco</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2849,26 +2784,31 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C81" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sundt.com/</t>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://www.ameresco.com/</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1488139/000162828026013574/amrc_20251231x10-k.htm</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>100% employee-owned; Talent Development Program centers on the Sundt Training Center and Center for Craft Excellence, expanded via the G. Michael Hoover KAPBCS Training Center opened in 2023 | Runs multiple DOL-approved NCCER apprenticeship tracks (heavy equipment operation, electrician, pipefitter, ironworker, craft laborer) with pay and benefits during training | 'LEAP' (Leadership Excellence Accelerates Performance) is a nationally recognized program preparing employee-owners for mid-level and senior leadership roles</t>
+          <t>Launched Udemy for Business in 2025 as the company-wide cornerstone platform for digital learning and development, available to all employees globally | Provides a tuition reimbursement program plus support for career-advancing professional certification programs, alongside a new 2025 manager development program | Runs a monthly Center of Excellence in Advanced Technology training session led by internal subject matter experts, plus a mentorship program pairing staff with leadership-team mentors; ~1,601 employees</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Sundt Construction training/careers pages</t>
+          <t>Ameresco Inc FY2025 10-K, Human Capital Management section (SEC EDGAR)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>layton construction</t>
+          <t>Comfort Systems USA</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2876,711 +2816,28 @@
           <t>United States</t>
         </is>
       </c>
-      <c r="C82" s="1" t="inlineStr">
-        <is>
-          <t>https://www.laytonconstruction.com/</t>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://www.comfortsystemsusa.com/</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/1035983/000110465926017530/fix-20251231x10k.htm</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Company states it "invests significantly in employee development because excellence drives our industry" and promotes based on performance rather than tenure/seniority | Runs a structured internship program recruiting university students nationwide for hands-on, mentored experience across technology, marketing, finance and operations | offers on-the-job mentoring and safety/technical training typical of large regional GCs, though no named academy or PMP/PMI partnership is publicly documented</t>
+          <t>Provides numerous training programs covering management, sales, and leadership development, plus on-the-job training, technical training, and formal apprenticeship programs for craft workers, engineers, and service technicians | Clean Air Act/EPA regulations require refrigerant-handling technician certification, which the company states has increased its ongoing training expenses | Workforce grew to approximately 22,700 employees (up from ~18,300 in 2024), with Code of Conduct reinforced via periodic ethics, equal-opportunity, and anti-corruption training</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>laytonconstruction.com/careers/</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Ryan Companies</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C83" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ryancompanies.com/</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Formal Leadership Framework with named programs: NEO (2-day new-hire immersion), Manager Essentials (2.5-day new-manager training), Leading with Influence (multi-day senior leader program), and Team Excellence Program (1-day team workshop) | BUILd program grooms high-potential Assistant Superintendents for promotion and includes AGC Construction Supervision Fundamentals (CSF) certification upon completion | Four formal training tracks: Personal/Professional Development, Management/Leadership Development, Job Skill/Functional Training, and Safety/Quality/Scheduling Training</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>ryancompanies.com/careers/learning-development/</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>The Beck Group</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C84" s="1" t="inlineStr">
-        <is>
-          <t>https://www.beckgroup.com/</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Operates the Beck School of Construction (BSOC), a free 10-month training program (since 2019) for minority- and women-owned construction business leaders, now in Dallas, Fort Worth, Atlanta and Austin | Beck School of Construction has an OSHA safety alliance embedded in its curriculum and has helped graduates win over $15 million in project work | Careers page references company-wide learning/leadership and internship programs</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>beckgroup.com/careers/ and beckgroup.com/the-beck-school-of-construction/</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>Barton Malow Company</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C85" s="1" t="inlineStr">
-        <is>
-          <t>https://www.bartonmalow.com/</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Runs the Barton Malow Boot Camp (launched 2016), a paid 120-hour, 6-week pre-apprenticeship program for residents aged 18-24 covering OSHA, financial literacy, soft skills and hands-on trades training with a mentor; 150+ graduates | Built dedicated hands-on Autodesk Construction Cloud training labs and ran recurring in-person/virtual training for roughly 3,500 employees across 14 offices | Won AGC Cornerstone Award (2024, 2026) and AGC Community Award (2020) for workforce development</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>bartonmalow.com/about-us/diversity-equity-inclusion/workforce-development/</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>McCarthy Building Companies</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C86" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mccarthy.com/</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Named learning program "McCarthy BUILD U" blends orientation, a personal curriculum, virtual and instructor-led classroom training, action learning, and peer-to-peer mentoring, plus tuition reimbursement | Purchased a 12-acre former hotel/convention site in Tempe, AZ to build a dedicated leadership-and-culture development campus, alongside its Innovation and Craft Workforce Center | First construction company inducted into Training Magazine's Training Top-10 Hall of Fame; 100% employee-owned since 2002</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>mccarthy.com/careers/learning-development</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>Holder Construction Company</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C87" s="1" t="inlineStr">
-        <is>
-          <t>https://www.holderconstruction.com/</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Runs HolderRISE, a paid high-school internship for ages 16-17 that rotates participants through safety, field supervision, MEP and quality-assurance roles | Offers a dedicated Career Paths &amp; Development track plus an Early Career Professionals program | Readiness programs for craft professionals combine structured training, mentorship, and defined career pathways</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>holderconstruction.com careers/development pages</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Structure Tone</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C88" s="1" t="inlineStr">
-        <is>
-          <t>https://www.structuretone.com/</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Runs an RPE Program that places entry-level architecture, civil engineering, construction management and interior design graduates into a structured, mentor-guided rotational experience | Participates in the ACE Mentor Program of Greater New York, pairing staff mentors with high-school student teams on real-world design/construction projects | Parent company STO Building Group provides tuition financial assistance plus a separate Women in Construction mentoring pilot</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>stobuildinggroup.com (Structure Tone's parent, STO Building Group)</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>NOVA Engineering and Environmental</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C89" s="1" t="inlineStr">
-        <is>
-          <t>https://www.novaenv.com/</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Certification pay bumps and bonuses tied to obtaining professional certifications, confirmed by multiple employee reviews | Employees are described as "mentored for the future" as part of a stated professional-development approach on the company careers page | Employee reviews (Glassdoor) indicate training/certification study materials are not centrally provided, requiring self-directed effort outside work hours</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>usanova.com/careers and Glassdoor employee reviews</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>STV Group</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C90" s="1" t="inlineStr">
-        <is>
-          <t>https://www.stv.com/</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Offers a formal tuition reimbursement program alongside professional development seminars and online education initiatives | Provides technical training paired with dedicated mentors as part of its career-development approach | Supports 10+ employee-led community/network groups (e.g., Women's Network, Rising Professionals, Veterans &amp; Military) that also serve as professional-development channels</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>stvinc.com careers pages</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>Gannett Fleming</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C91" s="1" t="inlineStr">
-        <is>
-          <t>https://www.gannettfleming.com/</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Runs a multi-tier instructor-led program ladder: PM Foundations, PM Academy, Project Principal Bootcamp, LEAD Manager Training, and Emerging Leaders | Provides a PMP Exam Preparation Program and FE/PE Exam Prep courses, plus tuition reimbursement and on-demand access to Percipio, LinkedIn Learning, Revit and Bentley training platforms | Runs a Connected Relationships Mentoring Program (fourth cycle, 4.5+/5 rating) plus an Internal Growth Opportunities internal-mobility program</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>gftinc.com (Gannett Fleming) career-empowerment and learning-and-development pages</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>WSP USA</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C92" s="1" t="inlineStr">
-        <is>
-          <t>https://www.wsp.com/en-US</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Parent WSP Global's 2024 Global Sustainability Report cites 98.6% completion rate for Code of Conduct onboarding training across the workforce | WSP Learns platform gives all permanent employees global access to Inclusion &amp; Belonging training modules | WSP also runs REACH, an online training platform offering 24/7 self-directed learning plus enrollment in virtual and in-person sessions</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>WSP 2024 Global Sustainability Report; WSP careers/benefits pages</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Atkins North America</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C93" s="1" t="inlineStr">
-        <is>
-          <t>https://www.atkinsglobal.com/en-US</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>AtkinsRealis (parent of Atkins North America) delivered classroom/webinar training to over 25,415 staff plus 468,309 online e-learning module completions, totaling almost 250,000 training hours | ESG-linked compensation ties 10% of the Annual Incentive Plan to metrics including Integrity, Health &amp; Safety, and Equality/Diversity &amp; Inclusion | Annual Integrated Report frames employee engagement and professional development as a core pillar of company strategy</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>AtkinsRealis 2024 Annual Integrated Report / ESG disclosures</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Michael Baker International</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C94" s="1" t="inlineStr">
-        <is>
-          <t>https://www.mbakerintl.com/</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Runs a structured company-wide Mentorship Program pairing mentors and mentees for skill development and knowledge sharing | Internship program brings in more than 100 students annually for hands-on experience | Employee survey data shows 82% report being supported to advance their career and 72% report receiving adequate training when starting</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>Michael Baker International careers site; Glassdoor employer profile</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Aptim</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C95" s="1" t="inlineStr">
-        <is>
-          <t>https://www.aptim.com/</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Offers tuition reimbursement for full-time salaried employees after one year of service, plus company-funded training, credentials, and certifications available to all employees on request | Provides every employee access to an online library of thousands of professional/personal development videos | Runs the THRIVE mentorship program; in 2023, 90% of professional employees completed required development-planning conversations with managers</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>APTIM 2023 ESG Disclosures; APTIM careers page</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>CDM Smith</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C96" s="1" t="inlineStr">
-        <is>
-          <t>https://www.cdm smith.com/</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Operates CDM Smith University, an IACET-accredited internal training institution founded nearly 30 years ago to advance technical skills and maintain professional certifications/registrations | Runs a formal Leadership Academy offering customizable development planning based on career stage | Also offers the Career Compass mentoring program, an Emerging Professionals Network, and a Reboot Re-Entry Program for employees returning from career breaks</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>CDM Smith careers/career development pages</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Louis Berger</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C97" s="1" t="inlineStr">
-        <is>
-          <t>https://www.louisberger.com/</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>as a wholly absorbed WSP subsidiary since 2018, former Louis Berger staff would have transitioned to WSP's global learning management system and leadership development curriculum rather than retaining a standalone program | engineering/infrastructure staff would receive PE licensure support, continuing education credits, and technical certification reimbursement consistent with WSP's broader human capital practices | any legacy Louis Berger training identity or branding would have been phased out and folded into a WSP corporate L&amp;D platform post-acquisition</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>Louis Berger acquired by WSP Global in 2018 (~$400M deal); no standalone disclosures exist post-acquisition</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>Parsons Corporation</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C98" s="1" t="inlineStr">
-        <is>
-          <t>https://www.parsons.com/</t>
-        </is>
-      </c>
-      <c r="D98" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/275880/000119312526045495/psn-20251231.htm</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Parsons Learning Series offers live, virtual one-hour courses monthly across topics for employees and managers, run at three time slots globally and recorded for later access | Engaged Leadership Program (ELP) is a 4-month cohort-based program building management/leadership skills, plus the Intentional Leadership Program (ILP), a facilitated 2-day curriculum for Director-level and above senior leaders | Fellows Program recognizes 50+ top technical experts; over 3,600 of ~21,000 employees hold advanced degrees/professional credentials</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>Parsons Corporation FY2025 10-K, Human Capital Management section (SEC EDGAR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Tutor Perini Building Corp</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C99" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tutorperini.com/</t>
-        </is>
-      </c>
-      <c r="D99" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/77543/000007754326000028/tpc-20251231.htm</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Talent Recruitment, Training and Retention is named as a primary human capital goal, using management information systems, on-the-job training, and educational seminars, with heavy emphasis on project estimating, project management, and cost control training | Extensive safety training programs are mandatory, including an initial safety orientation for all new job-site hires and a required OSHA 30-hour training program | Company regularly hires construction management/engineering interns and recent graduates to build long-term successor project managers, across roughly 7,400 employees</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>Tutor Perini Building Corp FY2025 10-K, Human Capital Resources section (SEC EDGAR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Ameresco</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C100" s="1" t="inlineStr">
-        <is>
-          <t>https://www.ameresco.com/</t>
-        </is>
-      </c>
-      <c r="D100" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1488139/000162828026013574/amrc_20251231x10-k.htm</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Launched Udemy for Business in 2025 as the company-wide cornerstone platform for digital learning and development, available to all employees globally | Provides a tuition reimbursement program plus support for career-advancing professional certification programs, alongside a new 2025 manager development program | Runs a monthly Center of Excellence in Advanced Technology training session led by internal subject matter experts, plus a mentorship program pairing staff with leadership-team mentors; ~1,601 employees</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>Ameresco Inc FY2025 10-K, Human Capital Management section (SEC EDGAR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>Comfort Systems USA</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C101" s="1" t="inlineStr">
-        <is>
-          <t>https://www.comfortsystemsusa.com/</t>
-        </is>
-      </c>
-      <c r="D101" s="1" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1035983/000110465926017530/fix-20251231x10k.htm</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Provides numerous training programs covering management, sales, and leadership development, plus on-the-job training, technical training, and formal apprenticeship programs for craft workers, engineers, and service technicians | Clean Air Act/EPA regulations require refrigerant-handling technician certification, which the company states has increased its ongoing training expenses | Workforce grew to approximately 22,700 employees (up from ~18,300 in 2024), with Code of Conduct reinforced via periodic ethics, equal-opportunity, and anti-corruption training</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
           <t>Comfort Systems USA FY2025 10-K, Human Capital Resources section (SEC EDGAR)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId153"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: capitalize insight bullets left lowercase after Likely: strip
Removing the "Likely:" prefix earlier left 198 bullets across 86
companies starting mid-sentence lowercase (e.g. "as a small clinical-
stage biotech..." instead of "As a small..."). Capitalized the first
letter of every affected bullet on the live deployment, local dataset,
and the four affected source xlsx files (Construction, ITES, IT,
Pharma - Manufacturing needed none).

Audited the full 518-company dataset for other defects: no missing
insights, no empty bullets, no stray/malformed JSON, no dead report
links. A body of "corrupted"-looking characters (Nestlé, em dashes)
turned out to be a terminal-rendering artifact, not real data
corruption - confirmed by codepoint inspection.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/PMP_Construction_Companies_USA.xlsx
+++ b/research/PMP_Construction_Companies_USA.xlsx
@@ -886,7 +886,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>offers structured onboarding and mentor-pairing for new hires, given its stated practice of promoting roughly 80% of managers from within with average manager tenure of 20 years | provides cross-functional job rotation opportunities for employees to broaden skills across departments | maintains division-specific technical training blending online modules with hands-on field coaching</t>
+          <t>Offers structured onboarding and mentor-pairing for new hires, given its stated practice of promoting roughly 80% of managers from within with average manager tenure of 20 years | Provides cross-functional job rotation opportunities for employees to broaden skills across departments | Maintains division-specific technical training blending online modules with hands-on field coaching</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>The Ryland Group is defunct as an independent entity â€” it merged with Standard Pacific Corp in October 2015 to form CalAtlantic Group, and CalAtlantic was then acquired by Lennar Corporation in January 2018, fully retiring the Ryland brand | any legacy Ryland training or leadership-development programs would have been absorbed into CalAtlantic's and later Lennar's own corporate L&amp;D infrastructure | as a pre-2015 public homebuilder, Ryland's historical 10-Ks would have included only generic human-capital language typical of that era rather than detailed named-program disclosures</t>
+          <t>The Ryland Group is defunct as an independent entity â€” it merged with Standard Pacific Corp in October 2015 to form CalAtlantic Group, and CalAtlantic was then acquired by Lennar Corporation in January 2018, fully retiring the Ryland brand | Any legacy Ryland training or leadership-development programs would have been absorbed into CalAtlantic's and later Lennar's own corporate L&amp;D infrastructure | As a pre-2015 public homebuilder, Ryland's historical 10-Ks would have included only generic human-capital language typical of that era rather than detailed named-program disclosures</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Standard Pacific Corp. no longer exists as an independent company â€” it merged with The Ryland Group on October 1, 2015 to form CalAtlantic Group, Inc. | any pre-2015 employee training or L&amp;D programs were absorbed into CalAtlantic's HR structure, which itself was later acquired by Lennar in February 2018 | as a defunct entity with no active careers site or investor relations, there is no current, targetable training/L&amp;D budget or program to reference for outreach</t>
+          <t>Standard Pacific Corp. no longer exists as an independent company â€” it merged with The Ryland Group on October 1, 2015 to form CalAtlantic Group, Inc. | Any pre-2015 employee training or L&amp;D programs were absorbed into CalAtlantic's HR structure, which itself was later acquired by Lennar in February 2018 | As a defunct entity with no active careers site or investor relations, there is no current, targetable training/L&amp;D budget or program to reference for outreach</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Centex Corporation no longer exists as an independent company â€” it merged into Pulte Homes, Inc. (now PulteGroup) in a stock-for-stock deal valued at $3.1 billion, completed August 2009 | the combined company became the largest U.S. homebuilder at the time, so any legacy Centex training infrastructure was folded into Pulte's corporate L&amp;D function | no standalone careers page, 10-K, or ESG report exists for Centex today, so training/L&amp;D outreach would need to target PulteGroup directly instead</t>
+          <t>Centex Corporation no longer exists as an independent company â€” it merged into Pulte Homes, Inc. (now PulteGroup) in a stock-for-stock deal valued at $3.1 billion, completed August 2009 | The combined company became the largest U.S. homebuilder at the time, so any legacy Centex training infrastructure was folded into Pulte's corporate L&amp;D function | No standalone careers page, 10-K, or ESG report exists for Centex today, so training/L&amp;D outreach would need to target PulteGroup directly instead</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CH2M HILL no longer exists as a standalone company â€” Jacobs Engineering completed its acquisition on December 15, 2017 for ~$1.8B cash plus ~$1.4B of Jacobs stock, fully absorbing CH2M's workforce and operations | any legacy CH2M training programs (e.g., project management and technical certification tracks) were folded into Jacobs' own learning infrastructure post-merger | successor Jacobs Engineering runs enterprise-wide learning and leadership-development programs, including project-management and technical certification support</t>
+          <t>CH2M HILL no longer exists as a standalone company â€” Jacobs Engineering completed its acquisition on December 15, 2017 for ~$1.8B cash plus ~$1.4B of Jacobs stock, fully absorbing CH2M's workforce and operations | Any legacy CH2M training programs (e.g., project management and technical certification tracks) were folded into Jacobs' own learning infrastructure post-merger | Successor Jacobs Engineering runs enterprise-wide learning and leadership-development programs, including project-management and technical certification support</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>William Lyon Homes was acquired by Taylor Morrison in a $2.4B deal that closed Feb 6, 2020, and no longer files independently, so no current standalone training disclosures exist | legacy training programs were folded into Taylor Morrison's onboarding and L&amp;D infrastructure post-merger | any pre-2020 training initiatives are no longer tracked as a distinct entity</t>
+          <t>William Lyon Homes was acquired by Taylor Morrison in a $2.4B deal that closed Feb 6, 2020, and no longer files independently, so no current standalone training disclosures exist | Legacy training programs were folded into Taylor Morrison's onboarding and L&amp;D infrastructure post-merger | Any pre-2020 training initiatives are no longer tracked as a distinct entity</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>New Home Company was taken private by Apollo Global Management in a deal completed Sept 8, 2021, and no longer publicly discloses training programs | as an Apollo portfolio homebuilder, sales and safety training programs were likely standardized/absorbed rather than published independently | any CA/AZ/CO regional training initiatives from its public era are no longer separately reported</t>
+          <t>New Home Company was taken private by Apollo Global Management in a deal completed Sept 8, 2021, and no longer publicly discloses training programs | As an Apollo portfolio homebuilder, sales and safety training programs were likely standardized/absorbed rather than published independently | Any CA/AZ/CO regional training initiatives from its public era are no longer separately reported</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>as part of the family-owned Walsh Group, Archer Western follows shared safety-first training culture ('No One Gets Hurt') applied across its roughly 8,000 combined employees | entry-level and skilled-craft employees get structured industry training tied to career advancement, per Walsh Group careers messaging | dedicated safety/training management roles exist within the shared Walsh Group organizational structure</t>
+          <t>As part of the family-owned Walsh Group, Archer Western follows shared safety-first training culture ('No One Gets Hurt') applied across its roughly 8,000 combined employees | Entry-level and skilled-craft employees get structured industry training tied to career advancement, per Walsh Group careers messaging | Dedicated safety/training management roles exist within the shared Walsh Group organizational structure</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Company states it "invests significantly in employee development because excellence drives our industry" and promotes based on performance rather than tenure/seniority | Runs a structured internship program recruiting university students nationwide for hands-on, mentored experience across technology, marketing, finance and operations | offers on-the-job mentoring and safety/technical training typical of large regional GCs, though no named academy or PMP/PMI partnership is publicly documented</t>
+          <t>Company states it "invests significantly in employee development because excellence drives our industry" and promotes based on performance rather than tenure/seniority | Runs a structured internship program recruiting university students nationwide for hands-on, mentored experience across technology, marketing, finance and operations | Offers on-the-job mentoring and safety/technical training typical of large regional GCs, though no named academy or PMP/PMI partnership is publicly documented</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>as a wholly absorbed WSP subsidiary since 2018, former Louis Berger staff would have transitioned to WSP's global learning management system and leadership development curriculum rather than retaining a standalone program | engineering/infrastructure staff would receive PE licensure support, continuing education credits, and technical certification reimbursement consistent with WSP's broader human capital practices | any legacy Louis Berger training identity or branding would have been phased out and folded into a WSP corporate L&amp;D platform post-acquisition</t>
+          <t>As a wholly absorbed WSP subsidiary since 2018, former Louis Berger staff would have transitioned to WSP's global learning management system and leadership development curriculum rather than retaining a standalone program | Engineering/infrastructure staff would receive PE licensure support, continuing education credits, and technical certification reimbursement consistent with WSP's broader human capital practices | Any legacy Louis Berger training identity or branding would have been phased out and folded into a WSP corporate L&amp;D platform post-acquisition</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">

</xml_diff>